<commit_message>
Completamos los ajustes y correcciones
</commit_message>
<xml_diff>
--- a/Memoria/library/mediciones auxiliares.xlsx
+++ b/Memoria/library/mediciones auxiliares.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Google Drive\Uni\TFG\Memoria\library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60552AEB-2B91-4A02-BCF4-54C1E2C1E491}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{091BBE06-EEB2-43B8-87C1-AC2F835B5339}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Euler" sheetId="3" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="77">
   <si>
     <t>Runge Kutta</t>
   </si>
@@ -69,9 +69,6 @@
   </si>
   <si>
     <t>Adams Bashford Moulton</t>
-  </si>
-  <si>
-    <t>Comparativa de métodos y tecnologías para Brusselator1D, neqn=100K</t>
   </si>
   <si>
     <t>Speedup</t>
@@ -268,6 +265,15 @@
   <si>
     <t>Grid2</t>
   </si>
+  <si>
+    <t>Comparativa de métodos y tecnologías para Brusselator1D, neqn=100K, y para simpleadvdiff</t>
+  </si>
+  <si>
+    <t>t(s)</t>
+  </si>
+  <si>
+    <t>OMP Componentes</t>
+  </si>
 </sst>
 </file>
 
@@ -432,6 +438,201 @@
     <cellStyle name="Normal 3" xfId="1" xr:uid="{F071A7C7-C907-4782-97BC-1691119DD71E}"/>
   </cellStyles>
   <dxfs count="32">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -850,201 +1051,6 @@
           <color theme="4" tint="0.39997558519241921"/>
         </bottom>
       </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -3679,7 +3685,7 @@
     <tableColumn id="7" xr3:uid="{64FA0956-3E24-4150-B966-D174B7BC073B}" name="Hebras"/>
     <tableColumn id="10" xr3:uid="{1B8321A3-89E7-440F-AC38-60832AF9D3BF}" name="T (s)"/>
     <tableColumn id="4" xr3:uid="{2A319FA1-3453-4EE4-B2DC-4F5247C2B6CA}" name="Speedup"/>
-    <tableColumn id="5" xr3:uid="{C8FBE361-944A-4D70-9B75-2CFCB1A1B454}" name="Efficiency" dataDxfId="22">
+    <tableColumn id="5" xr3:uid="{C8FBE361-944A-4D70-9B75-2CFCB1A1B454}" name="Efficiency" dataDxfId="31">
       <calculatedColumnFormula>Table1[[#This Row],[Speedup]]/Table1[[#This Row],[Hebras]]*100</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3688,6 +3694,20 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{E1C59661-95E7-4C50-B593-60AF4BF0419B}" name="Tabla9" displayName="Tabla9" ref="C3:E18" totalsRowShown="0">
+  <autoFilter ref="C3:E18" xr:uid="{E1C59661-95E7-4C50-B593-60AF4BF0419B}"/>
+  <tableColumns count="3">
+    <tableColumn id="10" xr3:uid="{386D6B24-9F12-4906-A98F-C1ECE9B2AF91}" name="T - CON"/>
+    <tableColumn id="12" xr3:uid="{BF967619-27A5-4370-8EB3-0CF9D0A5FB92}" name="T - SIN"/>
+    <tableColumn id="14" xr3:uid="{E8BDDCA8-85C9-47C8-B35D-4CDC5658DC19}" name="Sin/Con" dataDxfId="0">
+      <calculatedColumnFormula>Tabla9[[#This Row],[T - SIN]]/Tabla9[[#This Row],[T - CON]]</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{304C16FE-1A89-449E-B4E2-DA6D14937524}" name="Tabla10" displayName="Tabla10" ref="B4:D88" totalsRowShown="0">
   <autoFilter ref="B4:D88" xr:uid="{304C16FE-1A89-449E-B4E2-DA6D14937524}"/>
   <tableColumns count="3">
@@ -3699,7 +3719,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{A1DF3A69-E8A4-411B-83EC-4E166FFEA468}" name="Tabla11" displayName="Tabla11" ref="J4:L31" totalsRowShown="0">
   <autoFilter ref="J4:L31" xr:uid="{A1DF3A69-E8A4-411B-83EC-4E166FFEA468}"/>
   <tableColumns count="3">
@@ -3711,7 +3731,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{973BEA52-9B7C-4998-849D-398358C1B573}" name="Tabla12" displayName="Tabla12" ref="F4:H31" totalsRowShown="0">
   <autoFilter ref="F4:H31" xr:uid="{973BEA52-9B7C-4998-849D-398358C1B573}"/>
   <tableColumns count="3">
@@ -3723,7 +3743,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{816A0534-7E92-45A4-95E2-DE17D1227A63}" name="Tabla13" displayName="Tabla13" ref="O4:V17" totalsRowShown="0">
   <autoFilter ref="O4:V17" xr:uid="{816A0534-7E92-45A4-95E2-DE17D1227A63}"/>
   <tableColumns count="8">
@@ -3741,18 +3761,18 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{4C862F51-80EA-4323-A23D-AD6AF32D6737}" name="Table5" displayName="Table5" ref="A17:F23" totalsRowShown="0" tableBorderDxfId="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{4C862F51-80EA-4323-A23D-AD6AF32D6737}" name="Table5" displayName="Table5" ref="A17:F23" totalsRowShown="0" tableBorderDxfId="30">
   <autoFilter ref="A17:F23" xr:uid="{4C862F51-80EA-4323-A23D-AD6AF32D6737}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A18:D23">
     <sortCondition descending="1" ref="D17:D23"/>
   </sortState>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{969FCA7D-D340-4C13-86B2-C6EAC19CA12B}" name="Solver" dataDxfId="20"/>
-    <tableColumn id="2" xr3:uid="{F8648533-FD1A-4D6C-8084-2704645141D9}" name="Tipo" dataDxfId="19"/>
-    <tableColumn id="3" xr3:uid="{DC1BAEBC-A405-45AC-8E1D-FF0D7620EE8C}" name="Hebras" dataDxfId="18"/>
-    <tableColumn id="4" xr3:uid="{3D2F94AF-2C19-468F-80BC-25BE9607F57F}" name="T (s)" dataDxfId="17"/>
+    <tableColumn id="1" xr3:uid="{969FCA7D-D340-4C13-86B2-C6EAC19CA12B}" name="Solver" dataDxfId="29"/>
+    <tableColumn id="2" xr3:uid="{F8648533-FD1A-4D6C-8084-2704645141D9}" name="Tipo" dataDxfId="28"/>
+    <tableColumn id="3" xr3:uid="{DC1BAEBC-A405-45AC-8E1D-FF0D7620EE8C}" name="Hebras" dataDxfId="27"/>
+    <tableColumn id="4" xr3:uid="{3D2F94AF-2C19-468F-80BC-25BE9607F57F}" name="T (s)" dataDxfId="26"/>
     <tableColumn id="5" xr3:uid="{BF613CE6-6DEF-4C0B-848D-8F065FCF2C50}" name="Speedup"/>
-    <tableColumn id="6" xr3:uid="{0B73B7C0-235F-4E05-B847-5F924635199C}" name="Effiency" dataDxfId="16">
+    <tableColumn id="6" xr3:uid="{0B73B7C0-235F-4E05-B847-5F924635199C}" name="Effiency" dataDxfId="25">
       <calculatedColumnFormula>Table5[[#This Row],[Speedup]]/Table5[[#This Row],[Hebras]]*100</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3761,18 +3781,18 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{92F64B1B-7B7C-4525-B20C-2EFC812E8E5A}" name="Table4" displayName="Table4" ref="A9:F15" totalsRowShown="0" tableBorderDxfId="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{92F64B1B-7B7C-4525-B20C-2EFC812E8E5A}" name="Table4" displayName="Table4" ref="A9:F15" totalsRowShown="0" tableBorderDxfId="24">
   <autoFilter ref="A9:F15" xr:uid="{92F64B1B-7B7C-4525-B20C-2EFC812E8E5A}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A10:D15">
     <sortCondition descending="1" ref="D9:D15"/>
   </sortState>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{7672D6E0-6AC8-4B4D-A458-0BEE8A35C91C}" name="Solver" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{6C7C42B2-536F-4E04-830E-69EE87657A05}" name="Tipo" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{64021EE0-9E33-4FD5-83BD-34DA6D8320B7}" name="Hebras" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{397664F5-F154-4BCD-AD93-987F3D8C8EFE}" name="T (s)" dataDxfId="11"/>
+    <tableColumn id="1" xr3:uid="{7672D6E0-6AC8-4B4D-A458-0BEE8A35C91C}" name="Solver" dataDxfId="23"/>
+    <tableColumn id="2" xr3:uid="{6C7C42B2-536F-4E04-830E-69EE87657A05}" name="Tipo" dataDxfId="22"/>
+    <tableColumn id="3" xr3:uid="{64021EE0-9E33-4FD5-83BD-34DA6D8320B7}" name="Hebras" dataDxfId="21"/>
+    <tableColumn id="4" xr3:uid="{397664F5-F154-4BCD-AD93-987F3D8C8EFE}" name="T (s)" dataDxfId="20"/>
     <tableColumn id="5" xr3:uid="{417AEB65-89EB-4AD8-BE23-D32970ABEDB3}" name="Speedup"/>
-    <tableColumn id="6" xr3:uid="{BD17F5F8-C972-4C88-8F9D-3540C6C6AE0F}" name="Efficiency" dataDxfId="10">
+    <tableColumn id="6" xr3:uid="{BD17F5F8-C972-4C88-8F9D-3540C6C6AE0F}" name="Efficiency" dataDxfId="19">
       <calculatedColumnFormula>Table4[[#This Row],[Speedup]]/Table4[[#This Row],[Hebras]]*100</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3781,6 +3801,19 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{186076A2-FBD2-4EE7-8A1E-C4B2122C78FB}" name="Tabla14" displayName="Tabla14" ref="I4:L22" totalsRowShown="0">
+  <autoFilter ref="I4:L22" xr:uid="{186076A2-FBD2-4EE7-8A1E-C4B2122C78FB}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{036D236A-CB03-49C4-B738-BE410D43089B}" name="Solver"/>
+    <tableColumn id="2" xr3:uid="{FF42F9BC-7ED9-4788-ADC6-2835BD825437}" name="Tipo"/>
+    <tableColumn id="3" xr3:uid="{DE7EDE9F-AF7A-4557-A422-5F385DE6F3CA}" name="Hebras"/>
+    <tableColumn id="4" xr3:uid="{0498710B-FE7B-4168-BB94-20B57A6B5FCD}" name="t(s)"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8C8ECA13-2EB2-4FC1-85DE-E2A3D0878827}" name="Tabla2" displayName="Tabla2" ref="C3:H21" totalsRowShown="0">
   <autoFilter ref="C3:H21" xr:uid="{8C8ECA13-2EB2-4FC1-85DE-E2A3D0878827}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C4:F21">
@@ -3792,7 +3825,7 @@
     <tableColumn id="3" xr3:uid="{3A3C5E88-C7DA-483A-917E-BB271E1A560D}" name="Tipo"/>
     <tableColumn id="10" xr3:uid="{16A7936E-BB2A-4361-A80F-5CD098124D72}" name="T (s)"/>
     <tableColumn id="1" xr3:uid="{99669171-F1C7-4284-B05F-40B0C07B15FF}" name="Speedup"/>
-    <tableColumn id="2" xr3:uid="{0F99AB6F-95B0-48AC-AFFA-9572A938E9D5}" name="Effiency" dataDxfId="9">
+    <tableColumn id="2" xr3:uid="{0F99AB6F-95B0-48AC-AFFA-9572A938E9D5}" name="Effiency" dataDxfId="18">
       <calculatedColumnFormula>Tabla2[[#This Row],[Speedup]]/Tabla2[[#This Row],[Hebras]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3800,15 +3833,15 @@
 </table>
 </file>
 
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{500B26C9-CF13-4F25-BA27-B1B312614597}" name="Tabla3" displayName="Tabla3" ref="K3:O12" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7" tableBorderDxfId="6">
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{500B26C9-CF13-4F25-BA27-B1B312614597}" name="Tabla3" displayName="Tabla3" ref="K3:O12" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16" tableBorderDxfId="15">
   <autoFilter ref="K3:O12" xr:uid="{500B26C9-CF13-4F25-BA27-B1B312614597}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{9B87CB8C-71FB-48E7-ABD0-361458E1F0C5}" name="Hebras" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{7EE98D31-1E21-441D-ABE1-C50ADAD61A70}" name="neqn" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{147E8177-E9F7-4A21-8C6F-F807667557B0}" name="T (s)" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{9CC0064A-ACE5-4E3E-870C-8D7A7547540E}" name="Speedup" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{A4DD618E-02AE-479D-AF72-8E73365EF307}" name="Eficiencia" dataDxfId="1">
+    <tableColumn id="1" xr3:uid="{9B87CB8C-71FB-48E7-ABD0-361458E1F0C5}" name="Hebras" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{7EE98D31-1E21-441D-ABE1-C50ADAD61A70}" name="neqn" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{147E8177-E9F7-4A21-8C6F-F807667557B0}" name="T (s)" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{9CC0064A-ACE5-4E3E-870C-8D7A7547540E}" name="Speedup" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{A4DD618E-02AE-479D-AF72-8E73365EF307}" name="Eficiencia" dataDxfId="10">
       <calculatedColumnFormula>Tabla3[[#This Row],[Speedup]]/Tabla3[[#This Row],[Hebras]]*100</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3816,7 +3849,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{ED7CDD12-53B9-478E-8FA6-1644F23C7700}" name="Tabla6" displayName="Tabla6" ref="D3:G12" totalsRowShown="0">
   <autoFilter ref="D3:G12" xr:uid="{ED7CDD12-53B9-478E-8FA6-1644F23C7700}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="D4:F12">
@@ -3832,14 +3865,14 @@
 </table>
 </file>
 
-<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{BF881151-CBB8-40EC-B240-A88C073513E6}" name="Tabla7" displayName="Tabla7" ref="B3:E29" totalsRowShown="0">
   <autoFilter ref="B3:E29" xr:uid="{BF881151-CBB8-40EC-B240-A88C073513E6}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{644F7757-56D6-4333-9A04-BB025A3FA537}" name="Solver"/>
     <tableColumn id="9" xr3:uid="{7A4B951A-072B-4FA9-BB96-812FB6E68533}" name="neqn"/>
     <tableColumn id="10" xr3:uid="{27844286-B464-4C11-8051-BCFF52593894}" name="T (s)"/>
-    <tableColumn id="11" xr3:uid="{C4C270E6-294F-4C6C-9E30-CC46609C7C96}" name="ms/eq" dataDxfId="31">
+    <tableColumn id="11" xr3:uid="{C4C270E6-294F-4C6C-9E30-CC46609C7C96}" name="ms/eq" dataDxfId="9">
       <calculatedColumnFormula>Tabla7[[#This Row],[T (s)]]/Tabla7[[#This Row],[neqn]]*1000</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3847,33 +3880,19 @@
 </table>
 </file>
 
-<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{0C13DA08-D36E-4DC6-AD4D-C5ED3A2D2FFE}" name="Tabla8" displayName="Tabla8" ref="H3:P12" totalsRowShown="0" dataDxfId="30">
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{0C13DA08-D36E-4DC6-AD4D-C5ED3A2D2FFE}" name="Tabla8" displayName="Tabla8" ref="H3:P12" totalsRowShown="0" dataDxfId="8">
   <autoFilter ref="H3:P12" xr:uid="{0C13DA08-D36E-4DC6-AD4D-C5ED3A2D2FFE}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{932C3C52-A732-48FA-B5C5-2E96D1AF7393}" name="neqn"/>
     <tableColumn id="2" xr3:uid="{180E0420-BB3F-4A15-AA9C-8504B61074B7}" name="T (s)"/>
-    <tableColumn id="3" xr3:uid="{9CD8DE62-128C-4DC7-8194-28F682AB47BE}" name="ms/eq" dataDxfId="29"/>
-    <tableColumn id="4" xr3:uid="{1C3E6784-B380-4E71-BD53-644073AFAABA}" name="neqn2" dataDxfId="28"/>
-    <tableColumn id="5" xr3:uid="{61BCB526-EF0F-4CEE-92F7-BCE6C4B0BDFD}" name="T (s)3" dataDxfId="27"/>
-    <tableColumn id="6" xr3:uid="{B376E533-C766-4D62-969F-995271FAC762}" name="ms/eq4" dataDxfId="26"/>
-    <tableColumn id="7" xr3:uid="{93F3FE3F-20CE-4AD5-AA05-7DFC7DFBB20D}" name="neqn5" dataDxfId="25"/>
-    <tableColumn id="8" xr3:uid="{0DB727DE-811B-4C13-9A70-3781C9DD0690}" name="T (s)6" dataDxfId="24"/>
-    <tableColumn id="9" xr3:uid="{10AD593B-05BC-4C4D-9C4F-32785D7D5748}" name="ms/eq7" dataDxfId="23"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{E1C59661-95E7-4C50-B593-60AF4BF0419B}" name="Tabla9" displayName="Tabla9" ref="C3:E18" totalsRowShown="0">
-  <autoFilter ref="C3:E18" xr:uid="{E1C59661-95E7-4C50-B593-60AF4BF0419B}"/>
-  <tableColumns count="3">
-    <tableColumn id="10" xr3:uid="{386D6B24-9F12-4906-A98F-C1ECE9B2AF91}" name="T - CON"/>
-    <tableColumn id="12" xr3:uid="{BF967619-27A5-4370-8EB3-0CF9D0A5FB92}" name="T - SIN"/>
-    <tableColumn id="14" xr3:uid="{E8BDDCA8-85C9-47C8-B35D-4CDC5658DC19}" name="Sin/Con" dataDxfId="0">
-      <calculatedColumnFormula>Tabla9[[#This Row],[T - SIN]]/Tabla9[[#This Row],[T - CON]]</calculatedColumnFormula>
-    </tableColumn>
+    <tableColumn id="3" xr3:uid="{9CD8DE62-128C-4DC7-8194-28F682AB47BE}" name="ms/eq" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{1C3E6784-B380-4E71-BD53-644073AFAABA}" name="neqn2" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{61BCB526-EF0F-4CEE-92F7-BCE6C4B0BDFD}" name="T (s)3" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{B376E533-C766-4D62-969F-995271FAC762}" name="ms/eq4" dataDxfId="4"/>
+    <tableColumn id="7" xr3:uid="{93F3FE3F-20CE-4AD5-AA05-7DFC7DFBB20D}" name="neqn5" dataDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{0DB727DE-811B-4C13-9A70-3781C9DD0690}" name="T (s)6" dataDxfId="2"/>
+    <tableColumn id="9" xr3:uid="{10AD593B-05BC-4C4D-9C4F-32785D7D5748}" name="ms/eq7" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4151,12 +4170,12 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="H2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I2">
         <v>0.1</v>
@@ -4164,19 +4183,19 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -4416,15 +4435,18 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.28515625" customWidth="1"/>
+    <col min="9" max="9" width="23.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -4438,16 +4460,16 @@
         <v>6</v>
       </c>
       <c r="E1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F1" t="s">
         <v>10</v>
       </c>
-      <c r="F1" t="s">
-        <v>11</v>
-      </c>
       <c r="H1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -4468,7 +4490,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -4489,7 +4511,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>0</v>
       </c>
@@ -4510,8 +4532,20 @@
         <f>Table1[[#This Row],[Speedup]]/Table1[[#This Row],[Hebras]]*100</f>
         <v>93.282068414207814</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I4" t="s">
+        <v>3</v>
+      </c>
+      <c r="J4" t="s">
+        <v>4</v>
+      </c>
+      <c r="K4" t="s">
+        <v>5</v>
+      </c>
+      <c r="L4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>0</v>
       </c>
@@ -4532,8 +4566,20 @@
         <f>Table1[[#This Row],[Speedup]]/Table1[[#This Row],[Hebras]]*100</f>
         <v>103.84144865969402</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I5" t="s">
+        <v>0</v>
+      </c>
+      <c r="J5" t="s">
+        <v>76</v>
+      </c>
+      <c r="K5">
+        <v>1</v>
+      </c>
+      <c r="L5">
+        <v>1568.93</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>0</v>
       </c>
@@ -4554,8 +4600,20 @@
         <f>Table1[[#This Row],[Speedup]]/Table1[[#This Row],[Hebras]]*100</f>
         <v>79.34691599218533</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I6" t="s">
+        <v>0</v>
+      </c>
+      <c r="J6" t="s">
+        <v>1</v>
+      </c>
+      <c r="K6">
+        <v>1</v>
+      </c>
+      <c r="L6">
+        <v>345.55799999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>0</v>
       </c>
@@ -4576,8 +4634,34 @@
         <f>Table1[[#This Row],[Speedup]]/Table1[[#This Row],[Hebras]]*100</f>
         <v>53.544047757684645</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I7" t="s">
+        <v>0</v>
+      </c>
+      <c r="J7" t="s">
+        <v>76</v>
+      </c>
+      <c r="K7">
+        <v>4</v>
+      </c>
+      <c r="L7">
+        <v>432.42099999999999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="I8" t="s">
+        <v>0</v>
+      </c>
+      <c r="J8" t="s">
+        <v>1</v>
+      </c>
+      <c r="K8">
+        <v>4</v>
+      </c>
+      <c r="L8">
+        <v>98.190899999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -4591,13 +4675,25 @@
         <v>6</v>
       </c>
       <c r="E9" t="s">
+        <v>9</v>
+      </c>
+      <c r="F9" t="s">
         <v>10</v>
       </c>
-      <c r="F9" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I9" t="s">
+        <v>0</v>
+      </c>
+      <c r="J9" t="s">
+        <v>76</v>
+      </c>
+      <c r="K9">
+        <v>16</v>
+      </c>
+      <c r="L9">
+        <v>134.35499999999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>7</v>
       </c>
@@ -4617,8 +4713,20 @@
         <f>Table4[[#This Row],[Speedup]]/Table4[[#This Row],[Hebras]]*100</f>
         <v>100</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I10" t="s">
+        <v>0</v>
+      </c>
+      <c r="J10" t="s">
+        <v>1</v>
+      </c>
+      <c r="K10">
+        <v>16</v>
+      </c>
+      <c r="L10">
+        <v>78.525400000000005</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>7</v>
       </c>
@@ -4638,8 +4746,20 @@
         <f>Table4[[#This Row],[Speedup]]/Table4[[#This Row],[Hebras]]*100</f>
         <v>100</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I11" t="s">
+        <v>7</v>
+      </c>
+      <c r="J11" t="s">
+        <v>76</v>
+      </c>
+      <c r="K11">
+        <v>1</v>
+      </c>
+      <c r="L11">
+        <v>294.63900000000001</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
         <v>7</v>
       </c>
@@ -4660,8 +4780,20 @@
         <f>Table4[[#This Row],[Speedup]]/Table4[[#This Row],[Hebras]]*100</f>
         <v>98.523883514610802</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I12" t="s">
+        <v>7</v>
+      </c>
+      <c r="J12" t="s">
+        <v>1</v>
+      </c>
+      <c r="K12">
+        <v>1</v>
+      </c>
+      <c r="L12">
+        <v>175.83199999999999</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>7</v>
       </c>
@@ -4682,8 +4814,20 @@
         <f>Table4[[#This Row],[Speedup]]/Table4[[#This Row],[Hebras]]*100</f>
         <v>106.12227370928218</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I13" t="s">
+        <v>7</v>
+      </c>
+      <c r="J13" t="s">
+        <v>76</v>
+      </c>
+      <c r="K13">
+        <v>4</v>
+      </c>
+      <c r="L13">
+        <v>72.22</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="10" t="s">
         <v>7</v>
       </c>
@@ -4704,8 +4848,20 @@
         <f>Table4[[#This Row],[Speedup]]/Table4[[#This Row],[Hebras]]*100</f>
         <v>78.253997883837542</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I14" t="s">
+        <v>7</v>
+      </c>
+      <c r="J14" t="s">
+        <v>1</v>
+      </c>
+      <c r="K14">
+        <v>4</v>
+      </c>
+      <c r="L14">
+        <v>40.6982</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
         <v>7</v>
       </c>
@@ -4726,8 +4882,34 @@
         <f>Table4[[#This Row],[Speedup]]/Table4[[#This Row],[Hebras]]*100</f>
         <v>52.538133895704362</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="I15" t="s">
+        <v>7</v>
+      </c>
+      <c r="J15" t="s">
+        <v>76</v>
+      </c>
+      <c r="K15">
+        <v>16</v>
+      </c>
+      <c r="L15">
+        <v>34.569200000000002</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="I16" t="s">
+        <v>7</v>
+      </c>
+      <c r="J16" t="s">
+        <v>1</v>
+      </c>
+      <c r="K16">
+        <v>16</v>
+      </c>
+      <c r="L16">
+        <v>39.700499999999998</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>3</v>
       </c>
@@ -4741,13 +4923,25 @@
         <v>6</v>
       </c>
       <c r="E17" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F17" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="I17" t="s">
+        <v>8</v>
+      </c>
+      <c r="J17" t="s">
+        <v>76</v>
+      </c>
+      <c r="K17">
+        <v>1</v>
+      </c>
+      <c r="L17">
+        <v>1367.14</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>8</v>
       </c>
@@ -4767,8 +4961,20 @@
         <f>Table5[[#This Row],[Speedup]]/Table5[[#This Row],[Hebras]]*100</f>
         <v>100</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="I18" t="s">
+        <v>8</v>
+      </c>
+      <c r="J18" t="s">
+        <v>1</v>
+      </c>
+      <c r="K18">
+        <v>1</v>
+      </c>
+      <c r="L18">
+        <v>561.56399999999996</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>8</v>
       </c>
@@ -4788,8 +4994,20 @@
         <f>Table5[[#This Row],[Speedup]]/Table5[[#This Row],[Hebras]]*100</f>
         <v>100</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="I19" t="s">
+        <v>8</v>
+      </c>
+      <c r="J19" t="s">
+        <v>76</v>
+      </c>
+      <c r="K19">
+        <v>4</v>
+      </c>
+      <c r="L19">
+        <v>359.767</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>8</v>
       </c>
@@ -4810,8 +5028,20 @@
         <f>Table5[[#This Row],[Speedup]]/Table5[[#This Row],[Hebras]]*100</f>
         <v>56.4164826142027</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="I20" t="s">
+        <v>8</v>
+      </c>
+      <c r="J20" t="s">
+        <v>1</v>
+      </c>
+      <c r="K20">
+        <v>4</v>
+      </c>
+      <c r="L20">
+        <v>138.93100000000001</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>8</v>
       </c>
@@ -4832,8 +5062,20 @@
         <f>Table5[[#This Row],[Speedup]]/Table5[[#This Row],[Hebras]]*100</f>
         <v>101.17906113447393</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="I21" t="s">
+        <v>8</v>
+      </c>
+      <c r="J21" t="s">
+        <v>76</v>
+      </c>
+      <c r="K21">
+        <v>16</v>
+      </c>
+      <c r="L21">
+        <v>150.57900000000001</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>8</v>
       </c>
@@ -4854,8 +5096,20 @@
         <f>Table5[[#This Row],[Speedup]]/Table5[[#This Row],[Hebras]]*100</f>
         <v>76.770599740342945</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="I22" t="s">
+        <v>8</v>
+      </c>
+      <c r="J22" t="s">
+        <v>1</v>
+      </c>
+      <c r="K22">
+        <v>16</v>
+      </c>
+      <c r="L22">
+        <v>139.524</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
         <v>8</v>
       </c>
@@ -4879,10 +5133,11 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="3">
+  <tableParts count="4">
     <tablePart r:id="rId1"/>
     <tablePart r:id="rId2"/>
     <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
 </file>
@@ -4901,15 +5156,15 @@
   <sheetData>
     <row r="1" spans="3:15" x14ac:dyDescent="0.25">
       <c r="C1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K1" t="s">
         <v>14</v>
-      </c>
-      <c r="K1" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="3" spans="3:15" x14ac:dyDescent="0.25">
       <c r="C3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D3" t="s">
         <v>5</v>
@@ -4921,25 +5176,25 @@
         <v>6</v>
       </c>
       <c r="G3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="K3" t="s">
         <v>5</v>
       </c>
       <c r="L3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="M3" t="s">
         <v>6</v>
       </c>
       <c r="N3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="O3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="3:15" x14ac:dyDescent="0.25">
@@ -4950,7 +5205,7 @@
         <v>1</v>
       </c>
       <c r="E4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F4">
         <v>976.06100000000004</v>
@@ -4988,7 +5243,7 @@
         <v>1</v>
       </c>
       <c r="E5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F5">
         <v>2151.79</v>
@@ -5026,7 +5281,7 @@
         <v>4</v>
       </c>
       <c r="E6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F6">
         <v>263.08100000000002</v>
@@ -5065,7 +5320,7 @@
         <v>4</v>
       </c>
       <c r="E7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F7">
         <v>569.69299999999998</v>
@@ -5104,7 +5359,7 @@
         <v>16</v>
       </c>
       <c r="E8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F8">
         <v>180.66200000000001</v>
@@ -5143,7 +5398,7 @@
         <v>16</v>
       </c>
       <c r="E9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F9">
         <v>206.744</v>
@@ -5182,7 +5437,7 @@
         <v>1</v>
       </c>
       <c r="E10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F10">
         <v>1825.86</v>
@@ -5220,7 +5475,7 @@
         <v>1</v>
       </c>
       <c r="E11" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F11">
         <v>3970.37</v>
@@ -5258,7 +5513,7 @@
         <v>4</v>
       </c>
       <c r="E12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F12">
         <v>466.28199999999998</v>
@@ -5297,7 +5552,7 @@
         <v>4</v>
       </c>
       <c r="E13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F13">
         <v>1049.3499999999999</v>
@@ -5319,7 +5574,7 @@
         <v>16</v>
       </c>
       <c r="E14" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F14">
         <v>214.67</v>
@@ -5341,7 +5596,7 @@
         <v>16</v>
       </c>
       <c r="E15" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F15">
         <v>331.80900000000003</v>
@@ -5363,7 +5618,7 @@
         <v>1</v>
       </c>
       <c r="E16" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F16">
         <v>2692.79</v>
@@ -5384,7 +5639,7 @@
         <v>1</v>
       </c>
       <c r="E17" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F17">
         <v>5982.94</v>
@@ -5405,7 +5660,7 @@
         <v>4</v>
       </c>
       <c r="E18" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F18">
         <v>675.12300000000005</v>
@@ -5427,7 +5682,7 @@
         <v>4</v>
       </c>
       <c r="E19" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F19">
         <v>1593.61</v>
@@ -5449,7 +5704,7 @@
         <v>16</v>
       </c>
       <c r="E20" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F20">
         <v>264.40199999999999</v>
@@ -5471,7 +5726,7 @@
         <v>16</v>
       </c>
       <c r="E21" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F21">
         <v>445.08100000000002</v>
@@ -5508,7 +5763,7 @@
   <sheetData>
     <row r="1" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="4:7" x14ac:dyDescent="0.25">
@@ -5522,7 +5777,7 @@
         <v>6</v>
       </c>
       <c r="G3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="4:7" x14ac:dyDescent="0.25">
@@ -5530,7 +5785,7 @@
         <v>0</v>
       </c>
       <c r="E4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F4">
         <v>2531.0100000000002</v>
@@ -5545,7 +5800,7 @@
         <v>0</v>
       </c>
       <c r="E5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F5">
         <v>236.42</v>
@@ -5560,7 +5815,7 @@
         <v>0</v>
       </c>
       <c r="E6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F6">
         <v>77.1447</v>
@@ -5575,7 +5830,7 @@
         <v>7</v>
       </c>
       <c r="E7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F7">
         <v>847.87</v>
@@ -5589,7 +5844,7 @@
         <v>7</v>
       </c>
       <c r="E8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F8">
         <v>82.703999999999994</v>
@@ -5604,7 +5859,7 @@
         <v>7</v>
       </c>
       <c r="E9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F9">
         <v>23.554400000000001</v>
@@ -5619,7 +5874,7 @@
         <v>8</v>
       </c>
       <c r="E10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F10">
         <v>2692.79</v>
@@ -5633,7 +5888,7 @@
         <v>8</v>
       </c>
       <c r="E11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F11">
         <v>264.40199999999999</v>
@@ -5648,7 +5903,7 @@
         <v>8</v>
       </c>
       <c r="E12" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F12">
         <v>86.291600000000003</v>
@@ -5678,7 +5933,7 @@
   <sheetData>
     <row r="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="H1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="2:18" x14ac:dyDescent="0.25">
@@ -5697,40 +5952,40 @@
         <v>3</v>
       </c>
       <c r="C3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D3" t="s">
         <v>6</v>
       </c>
       <c r="E3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I3" t="s">
         <v>6</v>
       </c>
       <c r="J3" t="s">
+        <v>29</v>
+      </c>
+      <c r="K3" t="s">
         <v>30</v>
       </c>
-      <c r="K3" t="s">
+      <c r="L3" t="s">
         <v>31</v>
       </c>
-      <c r="L3" t="s">
+      <c r="M3" t="s">
         <v>32</v>
       </c>
-      <c r="M3" t="s">
+      <c r="N3" t="s">
         <v>33</v>
       </c>
-      <c r="N3" t="s">
+      <c r="O3" t="s">
         <v>34</v>
       </c>
-      <c r="O3" t="s">
+      <c r="P3" t="s">
         <v>35</v>
-      </c>
-      <c r="P3" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="4" spans="2:18" x14ac:dyDescent="0.25">
@@ -5757,7 +6012,7 @@
         <v>94.21</v>
       </c>
       <c r="K4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L4">
         <v>33.409999999999997</v>
@@ -5766,7 +6021,7 @@
         <v>0.55600000000000005</v>
       </c>
       <c r="N4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="O4">
         <v>246.38</v>
@@ -5799,7 +6054,7 @@
         <v>47.91</v>
       </c>
       <c r="K5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L5">
         <v>38.56</v>
@@ -5808,7 +6063,7 @@
         <v>0.48199999999999998</v>
       </c>
       <c r="N5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="O5">
         <v>291.95</v>
@@ -5832,7 +6087,7 @@
         <v>17.084399999999999</v>
       </c>
       <c r="H6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="I6">
         <v>17.079999999999998</v>
@@ -5841,7 +6096,7 @@
         <v>17.084</v>
       </c>
       <c r="K6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="L6">
         <v>43.4</v>
@@ -5850,7 +6105,7 @@
         <v>0.434</v>
       </c>
       <c r="N6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="O6">
         <v>335.23</v>
@@ -5874,7 +6129,7 @@
         <v>8.5485500000000005</v>
       </c>
       <c r="H7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I7">
         <v>17.09</v>
@@ -5883,7 +6138,7 @@
         <v>8.548</v>
       </c>
       <c r="K7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="L7">
         <v>68.540000000000006</v>
@@ -5892,7 +6147,7 @@
         <v>0.45600000000000002</v>
       </c>
       <c r="N7" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="O7">
         <v>379.27</v>
@@ -5916,7 +6171,7 @@
         <v>4.3003749999999998</v>
       </c>
       <c r="H8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I8">
         <v>17.2</v>
@@ -5925,7 +6180,7 @@
         <v>4.3003</v>
       </c>
       <c r="K8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="L8">
         <v>89.16</v>
@@ -5934,7 +6189,7 @@
         <v>0.44500000000000001</v>
       </c>
       <c r="N8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="O8">
         <v>423.52</v>
@@ -5958,7 +6213,7 @@
         <v>1.74387</v>
       </c>
       <c r="H9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I9">
         <v>17.43</v>
@@ -5967,7 +6222,7 @@
         <v>1.7430000000000001</v>
       </c>
       <c r="K9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="L9">
         <v>115.64</v>
@@ -5976,7 +6231,7 @@
         <v>0.46200000000000002</v>
       </c>
       <c r="N9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="O9">
         <v>469.07</v>
@@ -6000,7 +6255,7 @@
         <v>1.1150899999999999</v>
       </c>
       <c r="H10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I10">
         <v>22.3</v>
@@ -6009,7 +6264,7 @@
         <v>1.115</v>
       </c>
       <c r="K10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L10">
         <v>141.37</v>
@@ -6018,7 +6273,7 @@
         <v>0.47099999999999997</v>
       </c>
       <c r="N10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="O10">
         <v>702.06</v>
@@ -6042,7 +6297,7 @@
         <v>0.7860166666666667</v>
       </c>
       <c r="H11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I11">
         <v>23.58</v>
@@ -6051,7 +6306,7 @@
         <v>0.78600000000000003</v>
       </c>
       <c r="K11" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="L11">
         <v>173.56</v>
@@ -6060,7 +6315,7 @@
         <v>0.495</v>
       </c>
       <c r="N11" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="O11">
         <v>927.77</v>
@@ -6084,7 +6339,7 @@
         <v>0.70684499999999995</v>
       </c>
       <c r="H12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I12">
         <v>28.27</v>
@@ -6093,7 +6348,7 @@
         <v>0.70599999999999996</v>
       </c>
       <c r="K12" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="L12">
         <v>195.79</v>
@@ -6378,21 +6633,21 @@
   <sheetData>
     <row r="1" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B3" s="13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C3" t="s">
+        <v>62</v>
+      </c>
+      <c r="D3" t="s">
         <v>63</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>64</v>
-      </c>
-      <c r="E3" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.25">
@@ -6646,7 +6901,7 @@
   <sheetData>
     <row r="1" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" spans="2:22" x14ac:dyDescent="0.25">
@@ -6654,16 +6909,16 @@
         <v>4</v>
       </c>
       <c r="C4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D4" t="s">
         <v>6</v>
       </c>
       <c r="F4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H4" t="s">
         <v>6</v>
@@ -6672,39 +6927,39 @@
         <v>4</v>
       </c>
       <c r="K4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="L4" t="s">
         <v>6</v>
       </c>
       <c r="O4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="P4" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>69</v>
+      </c>
+      <c r="R4" t="s">
+        <v>68</v>
+      </c>
+      <c r="S4" t="s">
+        <v>30</v>
+      </c>
+      <c r="T4" t="s">
         <v>71</v>
       </c>
-      <c r="Q4" t="s">
-        <v>70</v>
-      </c>
-      <c r="R4" t="s">
-        <v>69</v>
-      </c>
-      <c r="S4" t="s">
-        <v>31</v>
-      </c>
-      <c r="T4" t="s">
+      <c r="U4" t="s">
         <v>72</v>
       </c>
-      <c r="U4" t="s">
+      <c r="V4" t="s">
         <v>73</v>
-      </c>
-      <c r="V4" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="5" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C5">
         <v>200</v>
@@ -6713,7 +6968,7 @@
         <v>4.2511799999999997</v>
       </c>
       <c r="F5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G5">
         <v>200</v>
@@ -6722,7 +6977,7 @@
         <v>4.2739500000000001</v>
       </c>
       <c r="J5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K5">
         <v>200</v>
@@ -6757,7 +7012,7 @@
     </row>
     <row r="6" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C6">
         <v>400</v>
@@ -6766,7 +7021,7 @@
         <v>4.3825000000000003</v>
       </c>
       <c r="F6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G6">
         <v>400</v>
@@ -6775,7 +7030,7 @@
         <v>4.4763099999999998</v>
       </c>
       <c r="J6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K6">
         <v>400</v>
@@ -6810,7 +7065,7 @@
     </row>
     <row r="7" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C7">
         <v>1000</v>
@@ -6819,7 +7074,7 @@
         <v>4.4242800000000004</v>
       </c>
       <c r="F7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G7">
         <v>1000</v>
@@ -6828,7 +7083,7 @@
         <v>4.4807300000000003</v>
       </c>
       <c r="J7" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K7">
         <v>1000</v>
@@ -6863,7 +7118,7 @@
     </row>
     <row r="8" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C8">
         <v>2000</v>
@@ -6872,7 +7127,7 @@
         <v>4.4725599999999996</v>
       </c>
       <c r="F8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G8">
         <v>2000</v>
@@ -6881,7 +7136,7 @@
         <v>4.4973900000000002</v>
       </c>
       <c r="J8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K8">
         <v>2000</v>
@@ -6916,7 +7171,7 @@
     </row>
     <row r="9" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C9">
         <v>4000</v>
@@ -6925,7 +7180,7 @@
         <v>4.5078199999999997</v>
       </c>
       <c r="F9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G9">
         <v>4000</v>
@@ -6934,7 +7189,7 @@
         <v>4.5514799999999997</v>
       </c>
       <c r="J9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K9">
         <v>4000</v>
@@ -6969,7 +7224,7 @@
     </row>
     <row r="10" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C10">
         <v>10000</v>
@@ -6978,7 +7233,7 @@
         <v>4.64262</v>
       </c>
       <c r="F10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G10">
         <v>10000</v>
@@ -6987,7 +7242,7 @@
         <v>4.7199299999999997</v>
       </c>
       <c r="J10" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K10">
         <v>10000</v>
@@ -7022,7 +7277,7 @@
     </row>
     <row r="11" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C11">
         <v>20000</v>
@@ -7031,7 +7286,7 @@
         <v>6.0775300000000003</v>
       </c>
       <c r="F11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G11">
         <v>20000</v>
@@ -7040,7 +7295,7 @@
         <v>6.194</v>
       </c>
       <c r="J11" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K11">
         <v>20000</v>
@@ -7075,7 +7330,7 @@
     </row>
     <row r="12" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C12">
         <v>30000</v>
@@ -7084,7 +7339,7 @@
         <v>6.4583899999999996</v>
       </c>
       <c r="F12" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G12">
         <v>40000</v>
@@ -7093,7 +7348,7 @@
         <v>7.7135699999999998</v>
       </c>
       <c r="J12" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K12">
         <v>40000</v>
@@ -7128,7 +7383,7 @@
     </row>
     <row r="13" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C13">
         <v>40000</v>
@@ -7137,7 +7392,7 @@
         <v>7.6532600000000004</v>
       </c>
       <c r="F13" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G13">
         <v>80000</v>
@@ -7146,7 +7401,7 @@
         <v>10.548500000000001</v>
       </c>
       <c r="J13" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K13">
         <v>80000</v>
@@ -7181,7 +7436,7 @@
     </row>
     <row r="14" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C14">
         <v>60000</v>
@@ -7190,7 +7445,7 @@
         <v>9.4447200000000002</v>
       </c>
       <c r="F14" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G14">
         <v>100000</v>
@@ -7199,7 +7454,7 @@
         <v>12.061299999999999</v>
       </c>
       <c r="J14" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K14">
         <v>100000</v>
@@ -7234,7 +7489,7 @@
     </row>
     <row r="15" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C15">
         <v>80000</v>
@@ -7243,7 +7498,7 @@
         <v>10.9232</v>
       </c>
       <c r="F15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G15">
         <v>150000</v>
@@ -7252,7 +7507,7 @@
         <v>21.8507</v>
       </c>
       <c r="J15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K15">
         <v>150000</v>
@@ -7287,7 +7542,7 @@
     </row>
     <row r="16" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C16">
         <v>100000</v>
@@ -7296,7 +7551,7 @@
         <v>13.191000000000001</v>
       </c>
       <c r="F16" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G16">
         <v>200000</v>
@@ -7305,7 +7560,7 @@
         <v>29.034800000000001</v>
       </c>
       <c r="J16" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K16">
         <v>200000</v>
@@ -7340,7 +7595,7 @@
     </row>
     <row r="17" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C17">
         <v>150000</v>
@@ -7349,7 +7604,7 @@
         <v>23.0747</v>
       </c>
       <c r="F17" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G17">
         <v>250000</v>
@@ -7358,7 +7613,7 @@
         <v>37.765799999999999</v>
       </c>
       <c r="J17" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K17">
         <v>250000</v>
@@ -7393,7 +7648,7 @@
     </row>
     <row r="18" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C18">
         <v>200000</v>
@@ -7402,7 +7657,7 @@
         <v>30.912700000000001</v>
       </c>
       <c r="F18" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G18">
         <v>300000</v>
@@ -7411,7 +7666,7 @@
         <v>47.618600000000001</v>
       </c>
       <c r="J18" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K18">
         <v>300000</v>
@@ -7422,7 +7677,7 @@
     </row>
     <row r="19" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C19">
         <v>250000</v>
@@ -7431,7 +7686,7 @@
         <v>41.323999999999998</v>
       </c>
       <c r="F19" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G19">
         <v>350000</v>
@@ -7440,7 +7695,7 @@
         <v>56.924599999999998</v>
       </c>
       <c r="J19" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K19">
         <v>350000</v>
@@ -7451,7 +7706,7 @@
     </row>
     <row r="20" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C20">
         <v>300000</v>
@@ -7460,7 +7715,7 @@
         <v>49.077300000000001</v>
       </c>
       <c r="F20" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G20">
         <v>400000</v>
@@ -7469,7 +7724,7 @@
         <v>64.066100000000006</v>
       </c>
       <c r="J20" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K20">
         <v>400000</v>
@@ -7480,7 +7735,7 @@
     </row>
     <row r="21" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C21">
         <v>350000</v>
@@ -7489,7 +7744,7 @@
         <v>58.703600000000002</v>
       </c>
       <c r="F21" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G21">
         <v>500000</v>
@@ -7498,7 +7753,7 @@
         <v>79.241900000000001</v>
       </c>
       <c r="J21" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K21">
         <v>500000</v>
@@ -7509,7 +7764,7 @@
     </row>
     <row r="22" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C22">
         <v>400000</v>
@@ -7518,7 +7773,7 @@
         <v>64.316400000000002</v>
       </c>
       <c r="F22" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G22">
         <v>600000</v>
@@ -7527,7 +7782,7 @@
         <v>93.808400000000006</v>
       </c>
       <c r="J22" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K22">
         <v>600000</v>
@@ -7538,7 +7793,7 @@
     </row>
     <row r="23" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C23">
         <v>500000</v>
@@ -7547,7 +7802,7 @@
         <v>78.499799999999993</v>
       </c>
       <c r="F23" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G23">
         <v>700000</v>
@@ -7556,7 +7811,7 @@
         <v>108.27200000000001</v>
       </c>
       <c r="J23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K23">
         <v>700000</v>
@@ -7567,7 +7822,7 @@
     </row>
     <row r="24" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C24">
         <v>600000</v>
@@ -7576,7 +7831,7 @@
         <v>92.214299999999994</v>
       </c>
       <c r="F24" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G24">
         <v>800000</v>
@@ -7585,7 +7840,7 @@
         <v>122.247</v>
       </c>
       <c r="J24" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K24">
         <v>800000</v>
@@ -7596,7 +7851,7 @@
     </row>
     <row r="25" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C25">
         <v>700000</v>
@@ -7605,7 +7860,7 @@
         <v>108.71599999999999</v>
       </c>
       <c r="F25" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G25">
         <v>900000</v>
@@ -7614,7 +7869,7 @@
         <v>136.72999999999999</v>
       </c>
       <c r="J25" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K25">
         <v>900000</v>
@@ -7625,7 +7880,7 @@
     </row>
     <row r="26" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C26">
         <v>800000</v>
@@ -7634,7 +7889,7 @@
         <v>123.306</v>
       </c>
       <c r="F26" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G26">
         <v>1000000</v>
@@ -7643,7 +7898,7 @@
         <v>151.23500000000001</v>
       </c>
       <c r="J26" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K26">
         <v>1000000</v>
@@ -7654,7 +7909,7 @@
     </row>
     <row r="27" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C27">
         <v>900000</v>
@@ -7663,7 +7918,7 @@
         <v>137.59899999999999</v>
       </c>
       <c r="F27" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G27">
         <v>1200000</v>
@@ -7672,7 +7927,7 @@
         <v>179.84100000000001</v>
       </c>
       <c r="J27" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K27">
         <v>1200000</v>
@@ -7683,7 +7938,7 @@
     </row>
     <row r="28" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C28">
         <v>1000000</v>
@@ -7692,7 +7947,7 @@
         <v>152.18700000000001</v>
       </c>
       <c r="F28" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G28">
         <v>1400000</v>
@@ -7701,7 +7956,7 @@
         <v>208.619</v>
       </c>
       <c r="J28" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K28">
         <v>1400000</v>
@@ -7712,7 +7967,7 @@
     </row>
     <row r="29" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C29">
         <v>1200000</v>
@@ -7721,7 +7976,7 @@
         <v>180.57599999999999</v>
       </c>
       <c r="F29" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G29">
         <v>1600000</v>
@@ -7730,7 +7985,7 @@
         <v>237.40600000000001</v>
       </c>
       <c r="J29" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K29">
         <v>1600000</v>
@@ -7741,7 +7996,7 @@
     </row>
     <row r="30" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C30">
         <v>1400000</v>
@@ -7750,7 +8005,7 @@
         <v>209.34700000000001</v>
       </c>
       <c r="F30" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G30">
         <v>1800000</v>
@@ -7759,7 +8014,7 @@
         <v>266.38499999999999</v>
       </c>
       <c r="J30" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K30">
         <v>1800000</v>
@@ -7770,7 +8025,7 @@
     </row>
     <row r="31" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C31">
         <v>1500000</v>
@@ -7779,7 +8034,7 @@
         <v>227.02</v>
       </c>
       <c r="F31" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G31">
         <v>2000000</v>
@@ -7788,7 +8043,7 @@
         <v>294.94799999999998</v>
       </c>
       <c r="J31" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K31">
         <v>2000000</v>
@@ -7799,7 +8054,7 @@
     </row>
     <row r="32" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C32">
         <v>1600000</v>
@@ -7810,7 +8065,7 @@
     </row>
     <row r="33" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C33">
         <v>1800000</v>
@@ -7821,7 +8076,7 @@
     </row>
     <row r="34" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C34">
         <v>2000000</v>
@@ -7832,7 +8087,7 @@
     </row>
     <row r="35" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B35" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C35">
         <v>200</v>
@@ -7843,7 +8098,7 @@
     </row>
     <row r="36" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B36" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C36">
         <v>400</v>
@@ -7854,7 +8109,7 @@
     </row>
     <row r="37" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B37" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C37">
         <v>1000</v>
@@ -7865,7 +8120,7 @@
     </row>
     <row r="38" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B38" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C38">
         <v>2000</v>
@@ -7876,7 +8131,7 @@
     </row>
     <row r="39" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C39">
         <v>4000</v>
@@ -7887,7 +8142,7 @@
     </row>
     <row r="40" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B40" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C40">
         <v>10000</v>
@@ -7898,7 +8153,7 @@
     </row>
     <row r="41" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B41" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C41">
         <v>20000</v>
@@ -7909,7 +8164,7 @@
     </row>
     <row r="42" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B42" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C42">
         <v>40000</v>
@@ -7920,7 +8175,7 @@
     </row>
     <row r="43" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B43" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C43">
         <v>80000</v>
@@ -7931,7 +8186,7 @@
     </row>
     <row r="44" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B44" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C44">
         <v>100000</v>
@@ -7942,7 +8197,7 @@
     </row>
     <row r="45" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B45" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C45">
         <v>150000</v>
@@ -7953,7 +8208,7 @@
     </row>
     <row r="46" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B46" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C46">
         <v>200000</v>
@@ -7964,7 +8219,7 @@
     </row>
     <row r="47" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B47" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C47">
         <v>250000</v>
@@ -7975,7 +8230,7 @@
     </row>
     <row r="48" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B48" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C48">
         <v>300000</v>
@@ -7986,7 +8241,7 @@
     </row>
     <row r="49" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B49" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C49">
         <v>350000</v>
@@ -7997,7 +8252,7 @@
     </row>
     <row r="50" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B50" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C50">
         <v>400000</v>
@@ -8008,7 +8263,7 @@
     </row>
     <row r="51" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B51" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C51">
         <v>500000</v>
@@ -8019,7 +8274,7 @@
     </row>
     <row r="52" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B52" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C52">
         <v>600000</v>
@@ -8030,7 +8285,7 @@
     </row>
     <row r="53" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B53" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C53">
         <v>700000</v>
@@ -8041,7 +8296,7 @@
     </row>
     <row r="54" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B54" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C54">
         <v>800000</v>
@@ -8052,7 +8307,7 @@
     </row>
     <row r="55" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B55" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C55">
         <v>900000</v>
@@ -8063,7 +8318,7 @@
     </row>
     <row r="56" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B56" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C56">
         <v>1000000</v>
@@ -8074,7 +8329,7 @@
     </row>
     <row r="57" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B57" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C57">
         <v>1200000</v>
@@ -8085,7 +8340,7 @@
     </row>
     <row r="58" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B58" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C58">
         <v>1400000</v>
@@ -8096,7 +8351,7 @@
     </row>
     <row r="59" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B59" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C59">
         <v>1600000</v>
@@ -8107,7 +8362,7 @@
     </row>
     <row r="60" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B60" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C60">
         <v>1800000</v>
@@ -8118,7 +8373,7 @@
     </row>
     <row r="61" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B61" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C61">
         <v>2000000</v>
@@ -8129,7 +8384,7 @@
     </row>
     <row r="62" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B62" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C62">
         <v>200</v>
@@ -8140,7 +8395,7 @@
     </row>
     <row r="63" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B63" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C63">
         <v>400</v>
@@ -8151,7 +8406,7 @@
     </row>
     <row r="64" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B64" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C64">
         <v>1000</v>
@@ -8162,7 +8417,7 @@
     </row>
     <row r="65" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B65" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C65">
         <v>2000</v>
@@ -8173,7 +8428,7 @@
     </row>
     <row r="66" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B66" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C66">
         <v>4000</v>
@@ -8184,7 +8439,7 @@
     </row>
     <row r="67" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B67" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C67">
         <v>10000</v>
@@ -8195,7 +8450,7 @@
     </row>
     <row r="68" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B68" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C68">
         <v>20000</v>
@@ -8206,7 +8461,7 @@
     </row>
     <row r="69" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B69" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C69">
         <v>40000</v>
@@ -8217,7 +8472,7 @@
     </row>
     <row r="70" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B70" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C70">
         <v>80000</v>
@@ -8228,7 +8483,7 @@
     </row>
     <row r="71" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B71" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C71">
         <v>100000</v>
@@ -8239,7 +8494,7 @@
     </row>
     <row r="72" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B72" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C72">
         <v>150000</v>
@@ -8250,7 +8505,7 @@
     </row>
     <row r="73" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B73" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C73">
         <v>200000</v>
@@ -8261,7 +8516,7 @@
     </row>
     <row r="74" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B74" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C74">
         <v>250000</v>
@@ -8272,7 +8527,7 @@
     </row>
     <row r="75" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B75" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C75">
         <v>300000</v>
@@ -8283,7 +8538,7 @@
     </row>
     <row r="76" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B76" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C76">
         <v>350000</v>
@@ -8294,7 +8549,7 @@
     </row>
     <row r="77" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B77" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C77">
         <v>400000</v>
@@ -8305,7 +8560,7 @@
     </row>
     <row r="78" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B78" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C78">
         <v>500000</v>
@@ -8316,7 +8571,7 @@
     </row>
     <row r="79" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B79" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C79">
         <v>600000</v>
@@ -8327,7 +8582,7 @@
     </row>
     <row r="80" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B80" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C80">
         <v>700000</v>
@@ -8338,7 +8593,7 @@
     </row>
     <row r="81" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B81" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C81">
         <v>800000</v>
@@ -8349,7 +8604,7 @@
     </row>
     <row r="82" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B82" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C82">
         <v>900000</v>
@@ -8360,7 +8615,7 @@
     </row>
     <row r="83" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B83" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C83">
         <v>1000000</v>
@@ -8371,7 +8626,7 @@
     </row>
     <row r="84" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B84" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C84">
         <v>1200000</v>
@@ -8382,7 +8637,7 @@
     </row>
     <row r="85" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B85" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C85">
         <v>1400000</v>
@@ -8393,7 +8648,7 @@
     </row>
     <row r="86" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B86" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C86">
         <v>1600000</v>
@@ -8404,7 +8659,7 @@
     </row>
     <row r="87" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B87" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C87">
         <v>1800000</v>
@@ -8415,7 +8670,7 @@
     </row>
     <row r="88" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B88" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C88">
         <v>2000000</v>

</xml_diff>

<commit_message>
Añado resumenes y objetivos
</commit_message>
<xml_diff>
--- a/Memoria/library/mediciones auxiliares.xlsx
+++ b/Memoria/library/mediciones auxiliares.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Google Drive\Uni\TFG\Memoria\library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{091BBE06-EEB2-43B8-87C1-AC2F835B5339}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4E93D6E-65F4-430F-8426-1278B3BD327A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Euler" sheetId="3" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="81">
   <si>
     <t>Runge Kutta</t>
   </si>
@@ -221,9 +221,6 @@
     <t>2M</t>
   </si>
   <si>
-    <t>Comparo RK y BR1D a través de distintos tamaños</t>
-  </si>
-  <si>
     <t>10K</t>
   </si>
   <si>
@@ -273,6 +270,21 @@
   </si>
   <si>
     <t>OMP Componentes</t>
+  </si>
+  <si>
+    <t>Comparo RK con ADV1D y BR1D a través de distintos tamaños</t>
+  </si>
+  <si>
+    <t>T (s)2</t>
+  </si>
+  <si>
+    <t>ms/eq2</t>
+  </si>
+  <si>
+    <t>neqn3</t>
+  </si>
+  <si>
+    <t>ms/eq3</t>
   </si>
 </sst>
 </file>
@@ -437,7 +449,10 @@
     <cellStyle name="Normal 2" xfId="2" xr:uid="{894E2A58-4AB2-4DD0-992A-D8EFC287A90D}"/>
     <cellStyle name="Normal 3" xfId="1" xr:uid="{F071A7C7-C907-4782-97BC-1691119DD71E}"/>
   </cellStyles>
-  <dxfs count="32">
+  <dxfs count="33">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -3685,7 +3700,7 @@
     <tableColumn id="7" xr3:uid="{64FA0956-3E24-4150-B966-D174B7BC073B}" name="Hebras"/>
     <tableColumn id="10" xr3:uid="{1B8321A3-89E7-440F-AC38-60832AF9D3BF}" name="T (s)"/>
     <tableColumn id="4" xr3:uid="{2A319FA1-3453-4EE4-B2DC-4F5247C2B6CA}" name="Speedup"/>
-    <tableColumn id="5" xr3:uid="{C8FBE361-944A-4D70-9B75-2CFCB1A1B454}" name="Efficiency" dataDxfId="31">
+    <tableColumn id="5" xr3:uid="{C8FBE361-944A-4D70-9B75-2CFCB1A1B454}" name="Efficiency" dataDxfId="32">
       <calculatedColumnFormula>Table1[[#This Row],[Speedup]]/Table1[[#This Row],[Hebras]]*100</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3694,12 +3709,44 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{E84F1AA3-4E90-4357-A9A3-E087AD695B92}" name="Tabla15" displayName="Tabla15" ref="G3:I29" totalsRowShown="0">
+  <autoFilter ref="G3:I29" xr:uid="{E84F1AA3-4E90-4357-A9A3-E087AD695B92}"/>
+  <tableColumns count="3">
+    <tableColumn id="9" xr3:uid="{1FB7F42F-A28A-415D-87DF-10147636C809}" name="neqn"/>
+    <tableColumn id="10" xr3:uid="{6B290550-A14F-4ED6-A0CB-28CFE477FCEE}" name="T (s)"/>
+    <tableColumn id="11" xr3:uid="{597C480E-1843-4915-8605-CF9C315F2D63}" name="ms/eq" dataDxfId="0">
+      <calculatedColumnFormula>Tabla15[[#This Row],[T (s)]]/Tabla15[[#This Row],[neqn]]*1000</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{E949A7C6-6E1E-413C-873F-68AF25297DF2}" name="Tabla16" displayName="Tabla16" ref="M16:U25" totalsRowShown="0">
+  <autoFilter ref="M16:U25" xr:uid="{E949A7C6-6E1E-413C-873F-68AF25297DF2}"/>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{E9B488FF-B52A-4052-8C3A-D4301FA7AB57}" name="neqn"/>
+    <tableColumn id="2" xr3:uid="{E70D4405-9CF2-4D72-BD7C-66B32DEFA8C8}" name="T (s)"/>
+    <tableColumn id="3" xr3:uid="{4E0AC869-9315-49EA-9D67-7CB514E7A481}" name="ms/eq"/>
+    <tableColumn id="4" xr3:uid="{7818AC8C-7334-41E5-823B-0321E63884E6}" name="neqn2"/>
+    <tableColumn id="5" xr3:uid="{C41A331F-1D98-48F7-9BE1-5B17DCF6221C}" name="T (s)2"/>
+    <tableColumn id="6" xr3:uid="{83C4B073-6F44-40D0-AB4C-F2C0392CC93A}" name="ms/eq2"/>
+    <tableColumn id="7" xr3:uid="{FE1D5C32-8FE7-4AD5-93A6-3DE319C4F0C0}" name="neqn3"/>
+    <tableColumn id="8" xr3:uid="{2C959683-0077-4596-BC4C-35B0D421A327}" name="T (s)3"/>
+    <tableColumn id="9" xr3:uid="{BA17556A-55CB-4776-92DE-26CF356532EE}" name="ms/eq3"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{E1C59661-95E7-4C50-B593-60AF4BF0419B}" name="Tabla9" displayName="Tabla9" ref="C3:E18" totalsRowShown="0">
   <autoFilter ref="C3:E18" xr:uid="{E1C59661-95E7-4C50-B593-60AF4BF0419B}"/>
   <tableColumns count="3">
     <tableColumn id="10" xr3:uid="{386D6B24-9F12-4906-A98F-C1ECE9B2AF91}" name="T - CON"/>
     <tableColumn id="12" xr3:uid="{BF967619-27A5-4370-8EB3-0CF9D0A5FB92}" name="T - SIN"/>
-    <tableColumn id="14" xr3:uid="{E8BDDCA8-85C9-47C8-B35D-4CDC5658DC19}" name="Sin/Con" dataDxfId="0">
+    <tableColumn id="14" xr3:uid="{E8BDDCA8-85C9-47C8-B35D-4CDC5658DC19}" name="Sin/Con" dataDxfId="1">
       <calculatedColumnFormula>Tabla9[[#This Row],[T - SIN]]/Tabla9[[#This Row],[T - CON]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3707,7 +3754,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{304C16FE-1A89-449E-B4E2-DA6D14937524}" name="Tabla10" displayName="Tabla10" ref="B4:D88" totalsRowShown="0">
   <autoFilter ref="B4:D88" xr:uid="{304C16FE-1A89-449E-B4E2-DA6D14937524}"/>
   <tableColumns count="3">
@@ -3719,7 +3766,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{A1DF3A69-E8A4-411B-83EC-4E166FFEA468}" name="Tabla11" displayName="Tabla11" ref="J4:L31" totalsRowShown="0">
   <autoFilter ref="J4:L31" xr:uid="{A1DF3A69-E8A4-411B-83EC-4E166FFEA468}"/>
   <tableColumns count="3">
@@ -3731,7 +3778,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{973BEA52-9B7C-4998-849D-398358C1B573}" name="Tabla12" displayName="Tabla12" ref="F4:H31" totalsRowShown="0">
   <autoFilter ref="F4:H31" xr:uid="{973BEA52-9B7C-4998-849D-398358C1B573}"/>
   <tableColumns count="3">
@@ -3743,7 +3790,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{816A0534-7E92-45A4-95E2-DE17D1227A63}" name="Tabla13" displayName="Tabla13" ref="O4:V17" totalsRowShown="0">
   <autoFilter ref="O4:V17" xr:uid="{816A0534-7E92-45A4-95E2-DE17D1227A63}"/>
   <tableColumns count="8">
@@ -3761,18 +3808,18 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{4C862F51-80EA-4323-A23D-AD6AF32D6737}" name="Table5" displayName="Table5" ref="A17:F23" totalsRowShown="0" tableBorderDxfId="30">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{4C862F51-80EA-4323-A23D-AD6AF32D6737}" name="Table5" displayName="Table5" ref="A17:F23" totalsRowShown="0" tableBorderDxfId="31">
   <autoFilter ref="A17:F23" xr:uid="{4C862F51-80EA-4323-A23D-AD6AF32D6737}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A18:D23">
     <sortCondition descending="1" ref="D17:D23"/>
   </sortState>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{969FCA7D-D340-4C13-86B2-C6EAC19CA12B}" name="Solver" dataDxfId="29"/>
-    <tableColumn id="2" xr3:uid="{F8648533-FD1A-4D6C-8084-2704645141D9}" name="Tipo" dataDxfId="28"/>
-    <tableColumn id="3" xr3:uid="{DC1BAEBC-A405-45AC-8E1D-FF0D7620EE8C}" name="Hebras" dataDxfId="27"/>
-    <tableColumn id="4" xr3:uid="{3D2F94AF-2C19-468F-80BC-25BE9607F57F}" name="T (s)" dataDxfId="26"/>
+    <tableColumn id="1" xr3:uid="{969FCA7D-D340-4C13-86B2-C6EAC19CA12B}" name="Solver" dataDxfId="30"/>
+    <tableColumn id="2" xr3:uid="{F8648533-FD1A-4D6C-8084-2704645141D9}" name="Tipo" dataDxfId="29"/>
+    <tableColumn id="3" xr3:uid="{DC1BAEBC-A405-45AC-8E1D-FF0D7620EE8C}" name="Hebras" dataDxfId="28"/>
+    <tableColumn id="4" xr3:uid="{3D2F94AF-2C19-468F-80BC-25BE9607F57F}" name="T (s)" dataDxfId="27"/>
     <tableColumn id="5" xr3:uid="{BF613CE6-6DEF-4C0B-848D-8F065FCF2C50}" name="Speedup"/>
-    <tableColumn id="6" xr3:uid="{0B73B7C0-235F-4E05-B847-5F924635199C}" name="Effiency" dataDxfId="25">
+    <tableColumn id="6" xr3:uid="{0B73B7C0-235F-4E05-B847-5F924635199C}" name="Effiency" dataDxfId="26">
       <calculatedColumnFormula>Table5[[#This Row],[Speedup]]/Table5[[#This Row],[Hebras]]*100</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3781,18 +3828,18 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{92F64B1B-7B7C-4525-B20C-2EFC812E8E5A}" name="Table4" displayName="Table4" ref="A9:F15" totalsRowShown="0" tableBorderDxfId="24">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{92F64B1B-7B7C-4525-B20C-2EFC812E8E5A}" name="Table4" displayName="Table4" ref="A9:F15" totalsRowShown="0" tableBorderDxfId="25">
   <autoFilter ref="A9:F15" xr:uid="{92F64B1B-7B7C-4525-B20C-2EFC812E8E5A}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A10:D15">
     <sortCondition descending="1" ref="D9:D15"/>
   </sortState>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{7672D6E0-6AC8-4B4D-A458-0BEE8A35C91C}" name="Solver" dataDxfId="23"/>
-    <tableColumn id="2" xr3:uid="{6C7C42B2-536F-4E04-830E-69EE87657A05}" name="Tipo" dataDxfId="22"/>
-    <tableColumn id="3" xr3:uid="{64021EE0-9E33-4FD5-83BD-34DA6D8320B7}" name="Hebras" dataDxfId="21"/>
-    <tableColumn id="4" xr3:uid="{397664F5-F154-4BCD-AD93-987F3D8C8EFE}" name="T (s)" dataDxfId="20"/>
+    <tableColumn id="1" xr3:uid="{7672D6E0-6AC8-4B4D-A458-0BEE8A35C91C}" name="Solver" dataDxfId="24"/>
+    <tableColumn id="2" xr3:uid="{6C7C42B2-536F-4E04-830E-69EE87657A05}" name="Tipo" dataDxfId="23"/>
+    <tableColumn id="3" xr3:uid="{64021EE0-9E33-4FD5-83BD-34DA6D8320B7}" name="Hebras" dataDxfId="22"/>
+    <tableColumn id="4" xr3:uid="{397664F5-F154-4BCD-AD93-987F3D8C8EFE}" name="T (s)" dataDxfId="21"/>
     <tableColumn id="5" xr3:uid="{417AEB65-89EB-4AD8-BE23-D32970ABEDB3}" name="Speedup"/>
-    <tableColumn id="6" xr3:uid="{BD17F5F8-C972-4C88-8F9D-3540C6C6AE0F}" name="Efficiency" dataDxfId="19">
+    <tableColumn id="6" xr3:uid="{BD17F5F8-C972-4C88-8F9D-3540C6C6AE0F}" name="Efficiency" dataDxfId="20">
       <calculatedColumnFormula>Table4[[#This Row],[Speedup]]/Table4[[#This Row],[Hebras]]*100</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3825,7 +3872,7 @@
     <tableColumn id="3" xr3:uid="{3A3C5E88-C7DA-483A-917E-BB271E1A560D}" name="Tipo"/>
     <tableColumn id="10" xr3:uid="{16A7936E-BB2A-4361-A80F-5CD098124D72}" name="T (s)"/>
     <tableColumn id="1" xr3:uid="{99669171-F1C7-4284-B05F-40B0C07B15FF}" name="Speedup"/>
-    <tableColumn id="2" xr3:uid="{0F99AB6F-95B0-48AC-AFFA-9572A938E9D5}" name="Effiency" dataDxfId="18">
+    <tableColumn id="2" xr3:uid="{0F99AB6F-95B0-48AC-AFFA-9572A938E9D5}" name="Effiency" dataDxfId="19">
       <calculatedColumnFormula>Tabla2[[#This Row],[Speedup]]/Tabla2[[#This Row],[Hebras]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3834,14 +3881,14 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{500B26C9-CF13-4F25-BA27-B1B312614597}" name="Tabla3" displayName="Tabla3" ref="K3:O12" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16" tableBorderDxfId="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{500B26C9-CF13-4F25-BA27-B1B312614597}" name="Tabla3" displayName="Tabla3" ref="K3:O12" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17" tableBorderDxfId="16">
   <autoFilter ref="K3:O12" xr:uid="{500B26C9-CF13-4F25-BA27-B1B312614597}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{9B87CB8C-71FB-48E7-ABD0-361458E1F0C5}" name="Hebras" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{7EE98D31-1E21-441D-ABE1-C50ADAD61A70}" name="neqn" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{147E8177-E9F7-4A21-8C6F-F807667557B0}" name="T (s)" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{9CC0064A-ACE5-4E3E-870C-8D7A7547540E}" name="Speedup" dataDxfId="11"/>
-    <tableColumn id="5" xr3:uid="{A4DD618E-02AE-479D-AF72-8E73365EF307}" name="Eficiencia" dataDxfId="10">
+    <tableColumn id="1" xr3:uid="{9B87CB8C-71FB-48E7-ABD0-361458E1F0C5}" name="Hebras" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{7EE98D31-1E21-441D-ABE1-C50ADAD61A70}" name="neqn" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{147E8177-E9F7-4A21-8C6F-F807667557B0}" name="T (s)" dataDxfId="13"/>
+    <tableColumn id="4" xr3:uid="{9CC0064A-ACE5-4E3E-870C-8D7A7547540E}" name="Speedup" dataDxfId="12"/>
+    <tableColumn id="5" xr3:uid="{A4DD618E-02AE-479D-AF72-8E73365EF307}" name="Eficiencia" dataDxfId="11">
       <calculatedColumnFormula>Tabla3[[#This Row],[Speedup]]/Tabla3[[#This Row],[Hebras]]*100</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3872,7 +3919,7 @@
     <tableColumn id="1" xr3:uid="{644F7757-56D6-4333-9A04-BB025A3FA537}" name="Solver"/>
     <tableColumn id="9" xr3:uid="{7A4B951A-072B-4FA9-BB96-812FB6E68533}" name="neqn"/>
     <tableColumn id="10" xr3:uid="{27844286-B464-4C11-8051-BCFF52593894}" name="T (s)"/>
-    <tableColumn id="11" xr3:uid="{C4C270E6-294F-4C6C-9E30-CC46609C7C96}" name="ms/eq" dataDxfId="9">
+    <tableColumn id="11" xr3:uid="{C4C270E6-294F-4C6C-9E30-CC46609C7C96}" name="ms/eq" dataDxfId="10">
       <calculatedColumnFormula>Tabla7[[#This Row],[T (s)]]/Tabla7[[#This Row],[neqn]]*1000</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3881,18 +3928,18 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{0C13DA08-D36E-4DC6-AD4D-C5ED3A2D2FFE}" name="Tabla8" displayName="Tabla8" ref="H3:P12" totalsRowShown="0" dataDxfId="8">
-  <autoFilter ref="H3:P12" xr:uid="{0C13DA08-D36E-4DC6-AD4D-C5ED3A2D2FFE}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{0C13DA08-D36E-4DC6-AD4D-C5ED3A2D2FFE}" name="Tabla8" displayName="Tabla8" ref="M3:U12" totalsRowShown="0" dataDxfId="9">
+  <autoFilter ref="M3:U12" xr:uid="{0C13DA08-D36E-4DC6-AD4D-C5ED3A2D2FFE}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{932C3C52-A732-48FA-B5C5-2E96D1AF7393}" name="neqn"/>
     <tableColumn id="2" xr3:uid="{180E0420-BB3F-4A15-AA9C-8504B61074B7}" name="T (s)"/>
-    <tableColumn id="3" xr3:uid="{9CD8DE62-128C-4DC7-8194-28F682AB47BE}" name="ms/eq" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{1C3E6784-B380-4E71-BD53-644073AFAABA}" name="neqn2" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{61BCB526-EF0F-4CEE-92F7-BCE6C4B0BDFD}" name="T (s)3" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{B376E533-C766-4D62-969F-995271FAC762}" name="ms/eq4" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{93F3FE3F-20CE-4AD5-AA05-7DFC7DFBB20D}" name="neqn5" dataDxfId="3"/>
-    <tableColumn id="8" xr3:uid="{0DB727DE-811B-4C13-9A70-3781C9DD0690}" name="T (s)6" dataDxfId="2"/>
-    <tableColumn id="9" xr3:uid="{10AD593B-05BC-4C4D-9C4F-32785D7D5748}" name="ms/eq7" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{9CD8DE62-128C-4DC7-8194-28F682AB47BE}" name="ms/eq" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{1C3E6784-B380-4E71-BD53-644073AFAABA}" name="neqn2" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{61BCB526-EF0F-4CEE-92F7-BCE6C4B0BDFD}" name="T (s)3" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{B376E533-C766-4D62-969F-995271FAC762}" name="ms/eq4" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{93F3FE3F-20CE-4AD5-AA05-7DFC7DFBB20D}" name="neqn5" dataDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{0DB727DE-811B-4C13-9A70-3781C9DD0690}" name="T (s)6" dataDxfId="3"/>
+    <tableColumn id="9" xr3:uid="{10AD593B-05BC-4C4D-9C4F-32785D7D5748}" name="ms/eq7" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4466,7 +4513,7 @@
         <v>10</v>
       </c>
       <c r="H1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
@@ -4542,7 +4589,7 @@
         <v>5</v>
       </c>
       <c r="L4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
@@ -4570,7 +4617,7 @@
         <v>0</v>
       </c>
       <c r="J5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="K5">
         <v>1</v>
@@ -4638,7 +4685,7 @@
         <v>0</v>
       </c>
       <c r="J7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="K7">
         <v>4</v>
@@ -4684,7 +4731,7 @@
         <v>0</v>
       </c>
       <c r="J9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="K9">
         <v>16</v>
@@ -4750,7 +4797,7 @@
         <v>7</v>
       </c>
       <c r="J11" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="K11">
         <v>1</v>
@@ -4818,7 +4865,7 @@
         <v>7</v>
       </c>
       <c r="J13" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="K13">
         <v>4</v>
@@ -4886,7 +4933,7 @@
         <v>7</v>
       </c>
       <c r="J15" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="K15">
         <v>16</v>
@@ -4932,7 +4979,7 @@
         <v>8</v>
       </c>
       <c r="J17" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="K17">
         <v>1</v>
@@ -4998,7 +5045,7 @@
         <v>8</v>
       </c>
       <c r="J19" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="K19">
         <v>4</v>
@@ -5066,7 +5113,7 @@
         <v>8</v>
       </c>
       <c r="J21" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="K21">
         <v>16</v>
@@ -5923,7 +5970,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61388887-C6C4-4F6F-8AD6-C9DE40C79BFF}">
-  <dimension ref="B1:R29"/>
+  <dimension ref="B1:U29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="23.5703125" bestFit="1" customWidth="1"/>
@@ -5931,23 +5978,21 @@
     <col min="7" max="7" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="H1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="2" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="J2" s="14"/>
-      <c r="K2" s="14"/>
-      <c r="L2" s="14"/>
-      <c r="M2" s="14"/>
-      <c r="N2" s="14"/>
+    <row r="1" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="M1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="2" spans="2:21" x14ac:dyDescent="0.25">
       <c r="O2" s="14"/>
       <c r="P2" s="14"/>
       <c r="Q2" s="14"/>
       <c r="R2" s="14"/>
-    </row>
-    <row r="3" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="S2" s="14"/>
+      <c r="T2" s="14"/>
+      <c r="U2" s="14"/>
+    </row>
+    <row r="3" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>3</v>
       </c>
@@ -5960,35 +6005,44 @@
       <c r="E3" t="s">
         <v>29</v>
       </c>
+      <c r="G3" t="s">
+        <v>12</v>
+      </c>
       <c r="H3" t="s">
+        <v>6</v>
+      </c>
+      <c r="I3" t="s">
+        <v>29</v>
+      </c>
+      <c r="M3" t="s">
         <v>12</v>
       </c>
-      <c r="I3" t="s">
+      <c r="N3" t="s">
         <v>6</v>
       </c>
-      <c r="J3" t="s">
+      <c r="O3" t="s">
         <v>29</v>
       </c>
-      <c r="K3" t="s">
+      <c r="P3" t="s">
         <v>30</v>
       </c>
-      <c r="L3" t="s">
+      <c r="Q3" t="s">
         <v>31</v>
       </c>
-      <c r="M3" t="s">
+      <c r="R3" t="s">
         <v>32</v>
       </c>
-      <c r="N3" t="s">
+      <c r="S3" t="s">
         <v>33</v>
       </c>
-      <c r="O3" t="s">
+      <c r="T3" t="s">
         <v>34</v>
       </c>
-      <c r="P3" t="s">
+      <c r="U3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>0</v>
       </c>
@@ -6002,35 +6056,45 @@
         <f>Tabla7[[#This Row],[T (s)]]/Tabla7[[#This Row],[neqn]]*1000</f>
         <v>94.21</v>
       </c>
+      <c r="G4">
+        <v>100</v>
+      </c>
       <c r="H4">
+        <v>21.426300000000001</v>
+      </c>
+      <c r="I4">
+        <f>Tabla15[[#This Row],[T (s)]]/Tabla15[[#This Row],[neqn]]*1000</f>
+        <v>214.26300000000001</v>
+      </c>
+      <c r="M4">
         <v>200</v>
       </c>
-      <c r="I4">
+      <c r="N4">
         <v>18.84</v>
       </c>
-      <c r="J4">
+      <c r="O4">
         <v>94.21</v>
       </c>
-      <c r="K4" t="s">
+      <c r="P4" t="s">
         <v>42</v>
       </c>
-      <c r="L4">
+      <c r="Q4">
         <v>33.409999999999997</v>
       </c>
-      <c r="M4">
+      <c r="R4">
         <v>0.55600000000000005</v>
       </c>
-      <c r="N4" t="s">
+      <c r="S4" t="s">
         <v>51</v>
       </c>
-      <c r="O4">
+      <c r="T4">
         <v>246.38</v>
       </c>
-      <c r="P4">
+      <c r="U4">
         <v>0.49199999999999999</v>
       </c>
     </row>
-    <row r="5" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>0</v>
       </c>
@@ -6044,35 +6108,45 @@
         <f>Tabla7[[#This Row],[T (s)]]/Tabla7[[#This Row],[neqn]]*1000</f>
         <v>47.91075</v>
       </c>
+      <c r="G5">
+        <v>200</v>
+      </c>
       <c r="H5">
+        <v>28.723600000000001</v>
+      </c>
+      <c r="I5">
+        <f>Tabla15[[#This Row],[T (s)]]/Tabla15[[#This Row],[neqn]]*1000</f>
+        <v>143.61799999999999</v>
+      </c>
+      <c r="M5">
         <v>400</v>
       </c>
-      <c r="I5">
+      <c r="N5">
         <v>19.16</v>
       </c>
-      <c r="J5">
+      <c r="O5">
         <v>47.91</v>
       </c>
-      <c r="K5" t="s">
+      <c r="P5" t="s">
         <v>43</v>
       </c>
-      <c r="L5">
+      <c r="Q5">
         <v>38.56</v>
       </c>
-      <c r="M5">
+      <c r="R5">
         <v>0.48199999999999998</v>
       </c>
-      <c r="N5" t="s">
+      <c r="S5" t="s">
         <v>52</v>
       </c>
-      <c r="O5">
+      <c r="T5">
         <v>291.95</v>
       </c>
-      <c r="P5">
+      <c r="U5">
         <v>0.48599999999999999</v>
       </c>
     </row>
-    <row r="6" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>0</v>
       </c>
@@ -6086,35 +6160,45 @@
         <f>Tabla7[[#This Row],[T (s)]]/Tabla7[[#This Row],[neqn]]*1000</f>
         <v>17.084399999999999</v>
       </c>
-      <c r="H6" t="s">
+      <c r="G6">
+        <v>500</v>
+      </c>
+      <c r="H6">
+        <v>31.041499999999999</v>
+      </c>
+      <c r="I6">
+        <f>Tabla15[[#This Row],[T (s)]]/Tabla15[[#This Row],[neqn]]*1000</f>
+        <v>62.082999999999998</v>
+      </c>
+      <c r="M6" t="s">
         <v>36</v>
       </c>
-      <c r="I6">
+      <c r="N6">
         <v>17.079999999999998</v>
       </c>
-      <c r="J6">
+      <c r="O6">
         <v>17.084</v>
       </c>
-      <c r="K6" t="s">
+      <c r="P6" t="s">
         <v>44</v>
       </c>
-      <c r="L6">
+      <c r="Q6">
         <v>43.4</v>
       </c>
-      <c r="M6">
+      <c r="R6">
         <v>0.434</v>
       </c>
-      <c r="N6" t="s">
+      <c r="S6" t="s">
         <v>53</v>
       </c>
-      <c r="O6">
+      <c r="T6">
         <v>335.23</v>
       </c>
-      <c r="P6">
+      <c r="U6">
         <v>0.47799999999999998</v>
       </c>
     </row>
-    <row r="7" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>0</v>
       </c>
@@ -6128,35 +6212,45 @@
         <f>Tabla7[[#This Row],[T (s)]]/Tabla7[[#This Row],[neqn]]*1000</f>
         <v>8.5485500000000005</v>
       </c>
-      <c r="H7" t="s">
+      <c r="G7">
+        <v>1000</v>
+      </c>
+      <c r="H7">
+        <v>30.878</v>
+      </c>
+      <c r="I7">
+        <f>Tabla15[[#This Row],[T (s)]]/Tabla15[[#This Row],[neqn]]*1000</f>
+        <v>30.878</v>
+      </c>
+      <c r="M7" t="s">
         <v>37</v>
       </c>
-      <c r="I7">
+      <c r="N7">
         <v>17.09</v>
       </c>
-      <c r="J7">
+      <c r="O7">
         <v>8.548</v>
       </c>
-      <c r="K7" t="s">
+      <c r="P7" t="s">
         <v>45</v>
       </c>
-      <c r="L7">
+      <c r="Q7">
         <v>68.540000000000006</v>
       </c>
-      <c r="M7">
+      <c r="R7">
         <v>0.45600000000000002</v>
       </c>
-      <c r="N7" t="s">
+      <c r="S7" t="s">
         <v>54</v>
       </c>
-      <c r="O7">
+      <c r="T7">
         <v>379.27</v>
       </c>
-      <c r="P7">
+      <c r="U7">
         <v>0.47399999999999998</v>
       </c>
     </row>
-    <row r="8" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>0</v>
       </c>
@@ -6170,35 +6264,45 @@
         <f>Tabla7[[#This Row],[T (s)]]/Tabla7[[#This Row],[neqn]]*1000</f>
         <v>4.3003749999999998</v>
       </c>
-      <c r="H8" t="s">
+      <c r="G8">
+        <v>2000</v>
+      </c>
+      <c r="H8">
+        <v>31.2256</v>
+      </c>
+      <c r="I8">
+        <f>Tabla15[[#This Row],[T (s)]]/Tabla15[[#This Row],[neqn]]*1000</f>
+        <v>15.6128</v>
+      </c>
+      <c r="M8" t="s">
         <v>38</v>
       </c>
-      <c r="I8">
+      <c r="N8">
         <v>17.2</v>
       </c>
-      <c r="J8">
+      <c r="O8">
         <v>4.3003</v>
       </c>
-      <c r="K8" t="s">
+      <c r="P8" t="s">
         <v>46</v>
       </c>
-      <c r="L8">
+      <c r="Q8">
         <v>89.16</v>
       </c>
-      <c r="M8">
+      <c r="R8">
         <v>0.44500000000000001</v>
       </c>
-      <c r="N8" t="s">
+      <c r="S8" t="s">
         <v>55</v>
       </c>
-      <c r="O8">
+      <c r="T8">
         <v>423.52</v>
       </c>
-      <c r="P8">
+      <c r="U8">
         <v>0.47</v>
       </c>
     </row>
-    <row r="9" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>0</v>
       </c>
@@ -6212,35 +6316,45 @@
         <f>Tabla7[[#This Row],[T (s)]]/Tabla7[[#This Row],[neqn]]*1000</f>
         <v>1.74387</v>
       </c>
-      <c r="H9" t="s">
-        <v>60</v>
+      <c r="G9">
+        <v>5000</v>
+      </c>
+      <c r="H9">
+        <v>31.218399999999999</v>
       </c>
       <c r="I9">
+        <f>Tabla15[[#This Row],[T (s)]]/Tabla15[[#This Row],[neqn]]*1000</f>
+        <v>6.2436799999999995</v>
+      </c>
+      <c r="M9" t="s">
+        <v>59</v>
+      </c>
+      <c r="N9">
         <v>17.43</v>
       </c>
-      <c r="J9">
+      <c r="O9">
         <v>1.7430000000000001</v>
       </c>
-      <c r="K9" t="s">
+      <c r="P9" t="s">
         <v>47</v>
       </c>
-      <c r="L9">
+      <c r="Q9">
         <v>115.64</v>
       </c>
-      <c r="M9">
+      <c r="R9">
         <v>0.46200000000000002</v>
       </c>
-      <c r="N9" t="s">
+      <c r="S9" t="s">
         <v>56</v>
       </c>
-      <c r="O9">
+      <c r="T9">
         <v>469.07</v>
       </c>
-      <c r="P9">
+      <c r="U9">
         <v>0.46899999999999997</v>
       </c>
     </row>
-    <row r="10" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>0</v>
       </c>
@@ -6254,35 +6368,45 @@
         <f>Tabla7[[#This Row],[T (s)]]/Tabla7[[#This Row],[neqn]]*1000</f>
         <v>1.1150899999999999</v>
       </c>
-      <c r="H10" t="s">
+      <c r="G10">
+        <v>10000</v>
+      </c>
+      <c r="H10">
+        <v>31.145700000000001</v>
+      </c>
+      <c r="I10">
+        <f>Tabla15[[#This Row],[T (s)]]/Tabla15[[#This Row],[neqn]]*1000</f>
+        <v>3.1145700000000001</v>
+      </c>
+      <c r="M10" t="s">
         <v>39</v>
       </c>
-      <c r="I10">
+      <c r="N10">
         <v>22.3</v>
       </c>
-      <c r="J10">
+      <c r="O10">
         <v>1.115</v>
       </c>
-      <c r="K10" t="s">
+      <c r="P10" t="s">
         <v>48</v>
       </c>
-      <c r="L10">
+      <c r="Q10">
         <v>141.37</v>
       </c>
-      <c r="M10">
+      <c r="R10">
         <v>0.47099999999999997</v>
       </c>
-      <c r="N10" t="s">
+      <c r="S10" t="s">
         <v>57</v>
       </c>
-      <c r="O10">
+      <c r="T10">
         <v>702.06</v>
       </c>
-      <c r="P10">
+      <c r="U10">
         <v>0.46800000000000003</v>
       </c>
     </row>
-    <row r="11" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>0</v>
       </c>
@@ -6296,35 +6420,45 @@
         <f>Tabla7[[#This Row],[T (s)]]/Tabla7[[#This Row],[neqn]]*1000</f>
         <v>0.7860166666666667</v>
       </c>
-      <c r="H11" t="s">
+      <c r="G11">
+        <v>15000</v>
+      </c>
+      <c r="H11">
+        <v>32.794499999999999</v>
+      </c>
+      <c r="I11">
+        <f>Tabla15[[#This Row],[T (s)]]/Tabla15[[#This Row],[neqn]]*1000</f>
+        <v>2.1863000000000001</v>
+      </c>
+      <c r="M11" t="s">
         <v>40</v>
       </c>
-      <c r="I11">
+      <c r="N11">
         <v>23.58</v>
       </c>
-      <c r="J11">
+      <c r="O11">
         <v>0.78600000000000003</v>
       </c>
-      <c r="K11" t="s">
+      <c r="P11" t="s">
         <v>50</v>
       </c>
-      <c r="L11">
+      <c r="Q11">
         <v>173.56</v>
       </c>
-      <c r="M11">
+      <c r="R11">
         <v>0.495</v>
       </c>
-      <c r="N11" t="s">
+      <c r="S11" t="s">
         <v>58</v>
       </c>
-      <c r="O11">
+      <c r="T11">
         <v>927.77</v>
       </c>
-      <c r="P11">
+      <c r="U11">
         <v>0.46300000000000002</v>
       </c>
     </row>
-    <row r="12" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>0</v>
       </c>
@@ -6338,26 +6472,36 @@
         <f>Tabla7[[#This Row],[T (s)]]/Tabla7[[#This Row],[neqn]]*1000</f>
         <v>0.70684499999999995</v>
       </c>
-      <c r="H12" t="s">
+      <c r="G12">
+        <v>20000</v>
+      </c>
+      <c r="H12">
+        <v>51.704099999999997</v>
+      </c>
+      <c r="I12">
+        <f>Tabla15[[#This Row],[T (s)]]/Tabla15[[#This Row],[neqn]]*1000</f>
+        <v>2.5852049999999998</v>
+      </c>
+      <c r="M12" t="s">
         <v>41</v>
       </c>
-      <c r="I12">
+      <c r="N12">
         <v>28.27</v>
       </c>
-      <c r="J12">
+      <c r="O12">
         <v>0.70599999999999996</v>
       </c>
-      <c r="K12" t="s">
+      <c r="P12" t="s">
         <v>49</v>
       </c>
-      <c r="L12">
+      <c r="Q12">
         <v>195.79</v>
       </c>
-      <c r="M12">
+      <c r="R12">
         <v>0.48899999999999999</v>
       </c>
     </row>
-    <row r="13" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>0</v>
       </c>
@@ -6371,8 +6515,18 @@
         <f>Tabla7[[#This Row],[T (s)]]/Tabla7[[#This Row],[neqn]]*1000</f>
         <v>0.55684166666666657</v>
       </c>
-    </row>
-    <row r="14" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="G13">
+        <v>30000</v>
+      </c>
+      <c r="H13">
+        <v>53.405799999999999</v>
+      </c>
+      <c r="I13">
+        <f>Tabla15[[#This Row],[T (s)]]/Tabla15[[#This Row],[neqn]]*1000</f>
+        <v>1.7801933333333333</v>
+      </c>
+    </row>
+    <row r="14" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>0</v>
       </c>
@@ -6386,8 +6540,18 @@
         <f>Tabla7[[#This Row],[T (s)]]/Tabla7[[#This Row],[neqn]]*1000</f>
         <v>0.48207250000000007</v>
       </c>
-    </row>
-    <row r="15" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="G14">
+        <v>40000</v>
+      </c>
+      <c r="H14">
+        <v>73.87</v>
+      </c>
+      <c r="I14">
+        <f>Tabla15[[#This Row],[T (s)]]/Tabla15[[#This Row],[neqn]]*1000</f>
+        <v>1.8467500000000001</v>
+      </c>
+    </row>
+    <row r="15" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>0</v>
       </c>
@@ -6401,8 +6565,18 @@
         <f>Tabla7[[#This Row],[T (s)]]/Tabla7[[#This Row],[neqn]]*1000</f>
         <v>0.43403700000000001</v>
       </c>
-    </row>
-    <row r="16" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="G15">
+        <v>50000</v>
+      </c>
+      <c r="H15">
+        <v>73.457300000000004</v>
+      </c>
+      <c r="I15">
+        <f>Tabla15[[#This Row],[T (s)]]/Tabla15[[#This Row],[neqn]]*1000</f>
+        <v>1.4691460000000001</v>
+      </c>
+    </row>
+    <row r="16" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>0</v>
       </c>
@@ -6416,8 +6590,45 @@
         <f>Tabla7[[#This Row],[T (s)]]/Tabla7[[#This Row],[neqn]]*1000</f>
         <v>0.45695600000000008</v>
       </c>
-    </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="G16">
+        <v>75000</v>
+      </c>
+      <c r="H16">
+        <v>115.03100000000001</v>
+      </c>
+      <c r="I16">
+        <f>Tabla15[[#This Row],[T (s)]]/Tabla15[[#This Row],[neqn]]*1000</f>
+        <v>1.5337466666666666</v>
+      </c>
+      <c r="M16" t="s">
+        <v>12</v>
+      </c>
+      <c r="N16" t="s">
+        <v>6</v>
+      </c>
+      <c r="O16" t="s">
+        <v>29</v>
+      </c>
+      <c r="P16" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>77</v>
+      </c>
+      <c r="R16" t="s">
+        <v>78</v>
+      </c>
+      <c r="S16" t="s">
+        <v>79</v>
+      </c>
+      <c r="T16" t="s">
+        <v>31</v>
+      </c>
+      <c r="U16" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="17" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>0</v>
       </c>
@@ -6431,8 +6642,46 @@
         <f>Tabla7[[#This Row],[T (s)]]/Tabla7[[#This Row],[neqn]]*1000</f>
         <v>0.4458105</v>
       </c>
-    </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="G17">
+        <v>100000</v>
+      </c>
+      <c r="H17">
+        <v>134.52500000000001</v>
+      </c>
+      <c r="I17">
+        <f>Tabla15[[#This Row],[T (s)]]/Tabla15[[#This Row],[neqn]]*1000</f>
+        <v>1.3452500000000001</v>
+      </c>
+      <c r="M17">
+        <v>50</v>
+      </c>
+      <c r="N17">
+        <v>27.43</v>
+      </c>
+      <c r="O17">
+        <f>Tabla16[[#This Row],[T (s)]]/Tabla16[[#This Row],[neqn]]*1000</f>
+        <v>548.6</v>
+      </c>
+      <c r="P17">
+        <v>20000</v>
+      </c>
+      <c r="Q17">
+        <v>51.704099999999997</v>
+      </c>
+      <c r="R17">
+        <v>2.5852049999999998</v>
+      </c>
+      <c r="S17">
+        <v>200000</v>
+      </c>
+      <c r="T17">
+        <v>270.13499999999999</v>
+      </c>
+      <c r="U17">
+        <v>1.3506750000000001</v>
+      </c>
+    </row>
+    <row r="18" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>0</v>
       </c>
@@ -6446,8 +6695,45 @@
         <f>Tabla7[[#This Row],[T (s)]]/Tabla7[[#This Row],[neqn]]*1000</f>
         <v>0.46257200000000004</v>
       </c>
-    </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="G18">
+        <v>125000</v>
+      </c>
+      <c r="H18">
+        <v>179.36500000000001</v>
+      </c>
+      <c r="I18">
+        <f>Tabla15[[#This Row],[T (s)]]/Tabla15[[#This Row],[neqn]]*1000</f>
+        <v>1.4349200000000002</v>
+      </c>
+      <c r="M18">
+        <v>100</v>
+      </c>
+      <c r="N18">
+        <v>21.426300000000001</v>
+      </c>
+      <c r="O18">
+        <v>214.26300000000001</v>
+      </c>
+      <c r="P18">
+        <v>30000</v>
+      </c>
+      <c r="Q18">
+        <v>53.405799999999999</v>
+      </c>
+      <c r="R18">
+        <v>1.7801933333333333</v>
+      </c>
+      <c r="S18">
+        <v>250000</v>
+      </c>
+      <c r="T18">
+        <v>340.20699999999999</v>
+      </c>
+      <c r="U18">
+        <v>1.3608279999999999</v>
+      </c>
+    </row>
+    <row r="19" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>0</v>
       </c>
@@ -6461,8 +6747,45 @@
         <f>Tabla7[[#This Row],[T (s)]]/Tabla7[[#This Row],[neqn]]*1000</f>
         <v>0.4712466666666667</v>
       </c>
-    </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="G19">
+        <v>150000</v>
+      </c>
+      <c r="H19">
+        <v>202.547</v>
+      </c>
+      <c r="I19">
+        <f>Tabla15[[#This Row],[T (s)]]/Tabla15[[#This Row],[neqn]]*1000</f>
+        <v>1.3503133333333333</v>
+      </c>
+      <c r="M19">
+        <v>200</v>
+      </c>
+      <c r="N19">
+        <v>28.723600000000001</v>
+      </c>
+      <c r="O19">
+        <v>143.61799999999999</v>
+      </c>
+      <c r="P19">
+        <v>40000</v>
+      </c>
+      <c r="Q19">
+        <v>73.87</v>
+      </c>
+      <c r="R19">
+        <v>1.8467500000000001</v>
+      </c>
+      <c r="S19">
+        <v>300000</v>
+      </c>
+      <c r="T19">
+        <v>411.625</v>
+      </c>
+      <c r="U19">
+        <v>1.3720833333333333</v>
+      </c>
+    </row>
+    <row r="20" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>0</v>
       </c>
@@ -6476,8 +6799,45 @@
         <f>Tabla7[[#This Row],[T (s)]]/Tabla7[[#This Row],[neqn]]*1000</f>
         <v>0.49589428571428568</v>
       </c>
-    </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="G20">
+        <v>175000</v>
+      </c>
+      <c r="H20">
+        <v>247.07400000000001</v>
+      </c>
+      <c r="I20">
+        <f>Tabla15[[#This Row],[T (s)]]/Tabla15[[#This Row],[neqn]]*1000</f>
+        <v>1.4118514285714285</v>
+      </c>
+      <c r="M20">
+        <v>500</v>
+      </c>
+      <c r="N20">
+        <v>31.041499999999999</v>
+      </c>
+      <c r="O20">
+        <v>62.082999999999998</v>
+      </c>
+      <c r="P20">
+        <v>50000</v>
+      </c>
+      <c r="Q20">
+        <v>73.457300000000004</v>
+      </c>
+      <c r="R20">
+        <v>1.4691460000000001</v>
+      </c>
+      <c r="S20">
+        <v>350000</v>
+      </c>
+      <c r="T20">
+        <v>484.81400000000002</v>
+      </c>
+      <c r="U20">
+        <v>1.385182857142857</v>
+      </c>
+    </row>
+    <row r="21" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
         <v>0</v>
       </c>
@@ -6491,8 +6851,45 @@
         <f>Tabla7[[#This Row],[T (s)]]/Tabla7[[#This Row],[neqn]]*1000</f>
         <v>0.48948250000000004</v>
       </c>
-    </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="G21">
+        <v>200000</v>
+      </c>
+      <c r="H21">
+        <v>270.13499999999999</v>
+      </c>
+      <c r="I21">
+        <f>Tabla15[[#This Row],[T (s)]]/Tabla15[[#This Row],[neqn]]*1000</f>
+        <v>1.3506750000000001</v>
+      </c>
+      <c r="M21">
+        <v>1000</v>
+      </c>
+      <c r="N21">
+        <v>30.878</v>
+      </c>
+      <c r="O21">
+        <v>30.878</v>
+      </c>
+      <c r="P21">
+        <v>75000</v>
+      </c>
+      <c r="Q21">
+        <v>115.03100000000001</v>
+      </c>
+      <c r="R21">
+        <v>1.5337466666666666</v>
+      </c>
+      <c r="S21">
+        <v>400000</v>
+      </c>
+      <c r="T21">
+        <v>542.48699999999997</v>
+      </c>
+      <c r="U21">
+        <v>1.3562175000000001</v>
+      </c>
+    </row>
+    <row r="22" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>0</v>
       </c>
@@ -6506,8 +6903,45 @@
         <f>Tabla7[[#This Row],[T (s)]]/Tabla7[[#This Row],[neqn]]*1000</f>
         <v>0.49277800000000005</v>
       </c>
-    </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="G22">
+        <v>250000</v>
+      </c>
+      <c r="H22">
+        <v>340.20699999999999</v>
+      </c>
+      <c r="I22">
+        <f>Tabla15[[#This Row],[T (s)]]/Tabla15[[#This Row],[neqn]]*1000</f>
+        <v>1.3608279999999999</v>
+      </c>
+      <c r="M22">
+        <v>2000</v>
+      </c>
+      <c r="N22">
+        <v>31.2256</v>
+      </c>
+      <c r="O22">
+        <v>15.6128</v>
+      </c>
+      <c r="P22">
+        <v>100000</v>
+      </c>
+      <c r="Q22">
+        <v>134.52500000000001</v>
+      </c>
+      <c r="R22">
+        <v>1.3452500000000001</v>
+      </c>
+      <c r="S22">
+        <v>450000</v>
+      </c>
+      <c r="T22">
+        <v>615.779</v>
+      </c>
+      <c r="U22">
+        <v>1.3683977777777778</v>
+      </c>
+    </row>
+    <row r="23" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
         <v>0</v>
       </c>
@@ -6521,8 +6955,45 @@
         <f>Tabla7[[#This Row],[T (s)]]/Tabla7[[#This Row],[neqn]]*1000</f>
         <v>0.48658500000000005</v>
       </c>
-    </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="G23">
+        <v>300000</v>
+      </c>
+      <c r="H23">
+        <v>411.625</v>
+      </c>
+      <c r="I23">
+        <f>Tabla15[[#This Row],[T (s)]]/Tabla15[[#This Row],[neqn]]*1000</f>
+        <v>1.3720833333333333</v>
+      </c>
+      <c r="M23">
+        <v>5000</v>
+      </c>
+      <c r="N23">
+        <v>31.218399999999999</v>
+      </c>
+      <c r="O23">
+        <v>6.2436799999999995</v>
+      </c>
+      <c r="P23">
+        <v>125000</v>
+      </c>
+      <c r="Q23">
+        <v>179.36500000000001</v>
+      </c>
+      <c r="R23">
+        <v>1.4349200000000002</v>
+      </c>
+      <c r="S23">
+        <v>500000</v>
+      </c>
+      <c r="T23">
+        <v>687.30799999999999</v>
+      </c>
+      <c r="U23">
+        <v>1.3746159999999998</v>
+      </c>
+    </row>
+    <row r="24" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
         <v>0</v>
       </c>
@@ -6536,8 +7007,45 @@
         <f>Tabla7[[#This Row],[T (s)]]/Tabla7[[#This Row],[neqn]]*1000</f>
         <v>0.47890714285714286</v>
       </c>
-    </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="G24">
+        <v>350000</v>
+      </c>
+      <c r="H24">
+        <v>484.81400000000002</v>
+      </c>
+      <c r="I24">
+        <f>Tabla15[[#This Row],[T (s)]]/Tabla15[[#This Row],[neqn]]*1000</f>
+        <v>1.385182857142857</v>
+      </c>
+      <c r="M24">
+        <v>10000</v>
+      </c>
+      <c r="N24">
+        <v>31.145700000000001</v>
+      </c>
+      <c r="O24">
+        <v>3.1145700000000001</v>
+      </c>
+      <c r="P24">
+        <v>150000</v>
+      </c>
+      <c r="Q24">
+        <v>202.547</v>
+      </c>
+      <c r="R24">
+        <v>1.3503133333333333</v>
+      </c>
+      <c r="S24">
+        <v>750000</v>
+      </c>
+      <c r="T24">
+        <v>1044.07</v>
+      </c>
+      <c r="U24">
+        <v>1.3920933333333332</v>
+      </c>
+    </row>
+    <row r="25" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
         <v>0</v>
       </c>
@@ -6551,8 +7059,45 @@
         <f>Tabla7[[#This Row],[T (s)]]/Tabla7[[#This Row],[neqn]]*1000</f>
         <v>0.47409125000000002</v>
       </c>
-    </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="G25">
+        <v>400000</v>
+      </c>
+      <c r="H25">
+        <v>542.48699999999997</v>
+      </c>
+      <c r="I25">
+        <f>Tabla15[[#This Row],[T (s)]]/Tabla15[[#This Row],[neqn]]*1000</f>
+        <v>1.3562175000000001</v>
+      </c>
+      <c r="M25">
+        <v>15000</v>
+      </c>
+      <c r="N25">
+        <v>32.794499999999999</v>
+      </c>
+      <c r="O25">
+        <v>2.1863000000000001</v>
+      </c>
+      <c r="P25">
+        <v>175000</v>
+      </c>
+      <c r="Q25">
+        <v>247.07400000000001</v>
+      </c>
+      <c r="R25">
+        <v>1.4118514285714285</v>
+      </c>
+      <c r="S25">
+        <v>1000000</v>
+      </c>
+      <c r="T25">
+        <v>1375.45</v>
+      </c>
+      <c r="U25">
+        <v>1.3754500000000001</v>
+      </c>
+    </row>
+    <row r="26" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
         <v>0</v>
       </c>
@@ -6566,8 +7111,18 @@
         <f>Tabla7[[#This Row],[T (s)]]/Tabla7[[#This Row],[neqn]]*1000</f>
         <v>0.47057888888888888</v>
       </c>
-    </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="G26">
+        <v>450000</v>
+      </c>
+      <c r="H26">
+        <v>615.779</v>
+      </c>
+      <c r="I26">
+        <f>Tabla15[[#This Row],[T (s)]]/Tabla15[[#This Row],[neqn]]*1000</f>
+        <v>1.3683977777777778</v>
+      </c>
+    </row>
+    <row r="27" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
         <v>0</v>
       </c>
@@ -6581,8 +7136,18 @@
         <f>Tabla7[[#This Row],[T (s)]]/Tabla7[[#This Row],[neqn]]*1000</f>
         <v>0.46907100000000007</v>
       </c>
-    </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="G27">
+        <v>500000</v>
+      </c>
+      <c r="H27">
+        <v>687.30799999999999</v>
+      </c>
+      <c r="I27">
+        <f>Tabla15[[#This Row],[T (s)]]/Tabla15[[#This Row],[neqn]]*1000</f>
+        <v>1.3746159999999998</v>
+      </c>
+    </row>
+    <row r="28" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
         <v>0</v>
       </c>
@@ -6596,8 +7161,18 @@
         <f>Tabla7[[#This Row],[T (s)]]/Tabla7[[#This Row],[neqn]]*1000</f>
         <v>0.46804533333333331</v>
       </c>
-    </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="G28">
+        <v>750000</v>
+      </c>
+      <c r="H28">
+        <v>1044.07</v>
+      </c>
+      <c r="I28">
+        <f>Tabla15[[#This Row],[T (s)]]/Tabla15[[#This Row],[neqn]]*1000</f>
+        <v>1.3920933333333332</v>
+      </c>
+    </row>
+    <row r="29" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
         <v>0</v>
       </c>
@@ -6611,12 +7186,24 @@
         <f>Tabla7[[#This Row],[T (s)]]/Tabla7[[#This Row],[neqn]]*1000</f>
         <v>0.46388749999999995</v>
       </c>
+      <c r="G29">
+        <v>1000000</v>
+      </c>
+      <c r="H29">
+        <v>1375.45</v>
+      </c>
+      <c r="I29">
+        <f>Tabla15[[#This Row],[T (s)]]/Tabla15[[#This Row],[neqn]]*1000</f>
+        <v>1.3754500000000001</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="2">
+  <tableParts count="4">
     <tablePart r:id="rId1"/>
     <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
 </file>
@@ -6633,7 +7220,7 @@
   <sheetData>
     <row r="1" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="2:5" x14ac:dyDescent="0.25">
@@ -6641,13 +7228,13 @@
         <v>12</v>
       </c>
       <c r="C3" t="s">
+        <v>61</v>
+      </c>
+      <c r="D3" t="s">
         <v>62</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>63</v>
-      </c>
-      <c r="E3" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.25">
@@ -6901,7 +7488,7 @@
   <sheetData>
     <row r="1" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" spans="2:22" x14ac:dyDescent="0.25">
@@ -6915,7 +7502,7 @@
         <v>6</v>
       </c>
       <c r="F4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G4" t="s">
         <v>12</v>
@@ -6936,30 +7523,30 @@
         <v>12</v>
       </c>
       <c r="P4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="Q4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="R4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="S4" t="s">
         <v>30</v>
       </c>
       <c r="T4" t="s">
+        <v>70</v>
+      </c>
+      <c r="U4" t="s">
         <v>71</v>
       </c>
-      <c r="U4" t="s">
+      <c r="V4" t="s">
         <v>72</v>
-      </c>
-      <c r="V4" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="5" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C5">
         <v>200</v>
@@ -6968,7 +7555,7 @@
         <v>4.2511799999999997</v>
       </c>
       <c r="F5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G5">
         <v>200</v>
@@ -6977,7 +7564,7 @@
         <v>4.2739500000000001</v>
       </c>
       <c r="J5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K5">
         <v>200</v>
@@ -7012,7 +7599,7 @@
     </row>
     <row r="6" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C6">
         <v>400</v>
@@ -7021,7 +7608,7 @@
         <v>4.3825000000000003</v>
       </c>
       <c r="F6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G6">
         <v>400</v>
@@ -7030,7 +7617,7 @@
         <v>4.4763099999999998</v>
       </c>
       <c r="J6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K6">
         <v>400</v>
@@ -7065,7 +7652,7 @@
     </row>
     <row r="7" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C7">
         <v>1000</v>
@@ -7074,7 +7661,7 @@
         <v>4.4242800000000004</v>
       </c>
       <c r="F7" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G7">
         <v>1000</v>
@@ -7083,7 +7670,7 @@
         <v>4.4807300000000003</v>
       </c>
       <c r="J7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K7">
         <v>1000</v>
@@ -7118,7 +7705,7 @@
     </row>
     <row r="8" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C8">
         <v>2000</v>
@@ -7127,7 +7714,7 @@
         <v>4.4725599999999996</v>
       </c>
       <c r="F8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G8">
         <v>2000</v>
@@ -7136,7 +7723,7 @@
         <v>4.4973900000000002</v>
       </c>
       <c r="J8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K8">
         <v>2000</v>
@@ -7171,7 +7758,7 @@
     </row>
     <row r="9" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C9">
         <v>4000</v>
@@ -7180,7 +7767,7 @@
         <v>4.5078199999999997</v>
       </c>
       <c r="F9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G9">
         <v>4000</v>
@@ -7189,7 +7776,7 @@
         <v>4.5514799999999997</v>
       </c>
       <c r="J9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K9">
         <v>4000</v>
@@ -7224,7 +7811,7 @@
     </row>
     <row r="10" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C10">
         <v>10000</v>
@@ -7233,7 +7820,7 @@
         <v>4.64262</v>
       </c>
       <c r="F10" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G10">
         <v>10000</v>
@@ -7242,7 +7829,7 @@
         <v>4.7199299999999997</v>
       </c>
       <c r="J10" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K10">
         <v>10000</v>
@@ -7277,7 +7864,7 @@
     </row>
     <row r="11" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C11">
         <v>20000</v>
@@ -7286,7 +7873,7 @@
         <v>6.0775300000000003</v>
       </c>
       <c r="F11" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G11">
         <v>20000</v>
@@ -7295,7 +7882,7 @@
         <v>6.194</v>
       </c>
       <c r="J11" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K11">
         <v>20000</v>
@@ -7330,7 +7917,7 @@
     </row>
     <row r="12" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C12">
         <v>30000</v>
@@ -7339,7 +7926,7 @@
         <v>6.4583899999999996</v>
       </c>
       <c r="F12" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G12">
         <v>40000</v>
@@ -7348,7 +7935,7 @@
         <v>7.7135699999999998</v>
       </c>
       <c r="J12" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K12">
         <v>40000</v>
@@ -7383,7 +7970,7 @@
     </row>
     <row r="13" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C13">
         <v>40000</v>
@@ -7392,7 +7979,7 @@
         <v>7.6532600000000004</v>
       </c>
       <c r="F13" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G13">
         <v>80000</v>
@@ -7401,7 +7988,7 @@
         <v>10.548500000000001</v>
       </c>
       <c r="J13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K13">
         <v>80000</v>
@@ -7436,7 +8023,7 @@
     </row>
     <row r="14" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C14">
         <v>60000</v>
@@ -7445,7 +8032,7 @@
         <v>9.4447200000000002</v>
       </c>
       <c r="F14" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G14">
         <v>100000</v>
@@ -7454,7 +8041,7 @@
         <v>12.061299999999999</v>
       </c>
       <c r="J14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K14">
         <v>100000</v>
@@ -7489,7 +8076,7 @@
     </row>
     <row r="15" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C15">
         <v>80000</v>
@@ -7498,7 +8085,7 @@
         <v>10.9232</v>
       </c>
       <c r="F15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G15">
         <v>150000</v>
@@ -7507,7 +8094,7 @@
         <v>21.8507</v>
       </c>
       <c r="J15" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K15">
         <v>150000</v>
@@ -7542,7 +8129,7 @@
     </row>
     <row r="16" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C16">
         <v>100000</v>
@@ -7551,7 +8138,7 @@
         <v>13.191000000000001</v>
       </c>
       <c r="F16" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G16">
         <v>200000</v>
@@ -7560,7 +8147,7 @@
         <v>29.034800000000001</v>
       </c>
       <c r="J16" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K16">
         <v>200000</v>
@@ -7595,7 +8182,7 @@
     </row>
     <row r="17" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C17">
         <v>150000</v>
@@ -7604,7 +8191,7 @@
         <v>23.0747</v>
       </c>
       <c r="F17" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G17">
         <v>250000</v>
@@ -7613,7 +8200,7 @@
         <v>37.765799999999999</v>
       </c>
       <c r="J17" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K17">
         <v>250000</v>
@@ -7648,7 +8235,7 @@
     </row>
     <row r="18" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C18">
         <v>200000</v>
@@ -7657,7 +8244,7 @@
         <v>30.912700000000001</v>
       </c>
       <c r="F18" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G18">
         <v>300000</v>
@@ -7666,7 +8253,7 @@
         <v>47.618600000000001</v>
       </c>
       <c r="J18" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K18">
         <v>300000</v>
@@ -7677,7 +8264,7 @@
     </row>
     <row r="19" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C19">
         <v>250000</v>
@@ -7686,7 +8273,7 @@
         <v>41.323999999999998</v>
       </c>
       <c r="F19" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G19">
         <v>350000</v>
@@ -7695,7 +8282,7 @@
         <v>56.924599999999998</v>
       </c>
       <c r="J19" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K19">
         <v>350000</v>
@@ -7706,7 +8293,7 @@
     </row>
     <row r="20" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C20">
         <v>300000</v>
@@ -7715,7 +8302,7 @@
         <v>49.077300000000001</v>
       </c>
       <c r="F20" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G20">
         <v>400000</v>
@@ -7724,7 +8311,7 @@
         <v>64.066100000000006</v>
       </c>
       <c r="J20" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K20">
         <v>400000</v>
@@ -7735,7 +8322,7 @@
     </row>
     <row r="21" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C21">
         <v>350000</v>
@@ -7744,7 +8331,7 @@
         <v>58.703600000000002</v>
       </c>
       <c r="F21" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G21">
         <v>500000</v>
@@ -7753,7 +8340,7 @@
         <v>79.241900000000001</v>
       </c>
       <c r="J21" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K21">
         <v>500000</v>
@@ -7764,7 +8351,7 @@
     </row>
     <row r="22" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C22">
         <v>400000</v>
@@ -7773,7 +8360,7 @@
         <v>64.316400000000002</v>
       </c>
       <c r="F22" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G22">
         <v>600000</v>
@@ -7782,7 +8369,7 @@
         <v>93.808400000000006</v>
       </c>
       <c r="J22" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K22">
         <v>600000</v>
@@ -7793,7 +8380,7 @@
     </row>
     <row r="23" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C23">
         <v>500000</v>
@@ -7802,7 +8389,7 @@
         <v>78.499799999999993</v>
       </c>
       <c r="F23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G23">
         <v>700000</v>
@@ -7811,7 +8398,7 @@
         <v>108.27200000000001</v>
       </c>
       <c r="J23" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K23">
         <v>700000</v>
@@ -7822,7 +8409,7 @@
     </row>
     <row r="24" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C24">
         <v>600000</v>
@@ -7831,7 +8418,7 @@
         <v>92.214299999999994</v>
       </c>
       <c r="F24" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G24">
         <v>800000</v>
@@ -7840,7 +8427,7 @@
         <v>122.247</v>
       </c>
       <c r="J24" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K24">
         <v>800000</v>
@@ -7851,7 +8438,7 @@
     </row>
     <row r="25" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C25">
         <v>700000</v>
@@ -7860,7 +8447,7 @@
         <v>108.71599999999999</v>
       </c>
       <c r="F25" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G25">
         <v>900000</v>
@@ -7869,7 +8456,7 @@
         <v>136.72999999999999</v>
       </c>
       <c r="J25" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K25">
         <v>900000</v>
@@ -7880,7 +8467,7 @@
     </row>
     <row r="26" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C26">
         <v>800000</v>
@@ -7889,7 +8476,7 @@
         <v>123.306</v>
       </c>
       <c r="F26" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G26">
         <v>1000000</v>
@@ -7898,7 +8485,7 @@
         <v>151.23500000000001</v>
       </c>
       <c r="J26" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K26">
         <v>1000000</v>
@@ -7909,7 +8496,7 @@
     </row>
     <row r="27" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C27">
         <v>900000</v>
@@ -7918,7 +8505,7 @@
         <v>137.59899999999999</v>
       </c>
       <c r="F27" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G27">
         <v>1200000</v>
@@ -7927,7 +8514,7 @@
         <v>179.84100000000001</v>
       </c>
       <c r="J27" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K27">
         <v>1200000</v>
@@ -7938,7 +8525,7 @@
     </row>
     <row r="28" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C28">
         <v>1000000</v>
@@ -7947,7 +8534,7 @@
         <v>152.18700000000001</v>
       </c>
       <c r="F28" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G28">
         <v>1400000</v>
@@ -7956,7 +8543,7 @@
         <v>208.619</v>
       </c>
       <c r="J28" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K28">
         <v>1400000</v>
@@ -7967,7 +8554,7 @@
     </row>
     <row r="29" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C29">
         <v>1200000</v>
@@ -7976,7 +8563,7 @@
         <v>180.57599999999999</v>
       </c>
       <c r="F29" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G29">
         <v>1600000</v>
@@ -7985,7 +8572,7 @@
         <v>237.40600000000001</v>
       </c>
       <c r="J29" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K29">
         <v>1600000</v>
@@ -7996,7 +8583,7 @@
     </row>
     <row r="30" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C30">
         <v>1400000</v>
@@ -8005,7 +8592,7 @@
         <v>209.34700000000001</v>
       </c>
       <c r="F30" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G30">
         <v>1800000</v>
@@ -8014,7 +8601,7 @@
         <v>266.38499999999999</v>
       </c>
       <c r="J30" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K30">
         <v>1800000</v>
@@ -8025,7 +8612,7 @@
     </row>
     <row r="31" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C31">
         <v>1500000</v>
@@ -8034,7 +8621,7 @@
         <v>227.02</v>
       </c>
       <c r="F31" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G31">
         <v>2000000</v>
@@ -8043,7 +8630,7 @@
         <v>294.94799999999998</v>
       </c>
       <c r="J31" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K31">
         <v>2000000</v>
@@ -8054,7 +8641,7 @@
     </row>
     <row r="32" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C32">
         <v>1600000</v>
@@ -8065,7 +8652,7 @@
     </row>
     <row r="33" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C33">
         <v>1800000</v>
@@ -8076,7 +8663,7 @@
     </row>
     <row r="34" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C34">
         <v>2000000</v>
@@ -8087,7 +8674,7 @@
     </row>
     <row r="35" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B35" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C35">
         <v>200</v>
@@ -8098,7 +8685,7 @@
     </row>
     <row r="36" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B36" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C36">
         <v>400</v>
@@ -8109,7 +8696,7 @@
     </row>
     <row r="37" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B37" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C37">
         <v>1000</v>
@@ -8120,7 +8707,7 @@
     </row>
     <row r="38" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B38" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C38">
         <v>2000</v>
@@ -8131,7 +8718,7 @@
     </row>
     <row r="39" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C39">
         <v>4000</v>
@@ -8142,7 +8729,7 @@
     </row>
     <row r="40" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B40" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C40">
         <v>10000</v>
@@ -8153,7 +8740,7 @@
     </row>
     <row r="41" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B41" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C41">
         <v>20000</v>
@@ -8164,7 +8751,7 @@
     </row>
     <row r="42" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B42" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C42">
         <v>40000</v>
@@ -8175,7 +8762,7 @@
     </row>
     <row r="43" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B43" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C43">
         <v>80000</v>
@@ -8186,7 +8773,7 @@
     </row>
     <row r="44" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B44" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C44">
         <v>100000</v>
@@ -8197,7 +8784,7 @@
     </row>
     <row r="45" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B45" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C45">
         <v>150000</v>
@@ -8208,7 +8795,7 @@
     </row>
     <row r="46" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B46" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C46">
         <v>200000</v>
@@ -8219,7 +8806,7 @@
     </row>
     <row r="47" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C47">
         <v>250000</v>
@@ -8230,7 +8817,7 @@
     </row>
     <row r="48" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B48" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C48">
         <v>300000</v>
@@ -8241,7 +8828,7 @@
     </row>
     <row r="49" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B49" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C49">
         <v>350000</v>
@@ -8252,7 +8839,7 @@
     </row>
     <row r="50" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B50" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C50">
         <v>400000</v>
@@ -8263,7 +8850,7 @@
     </row>
     <row r="51" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B51" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C51">
         <v>500000</v>
@@ -8274,7 +8861,7 @@
     </row>
     <row r="52" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B52" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C52">
         <v>600000</v>
@@ -8285,7 +8872,7 @@
     </row>
     <row r="53" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B53" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C53">
         <v>700000</v>
@@ -8296,7 +8883,7 @@
     </row>
     <row r="54" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B54" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C54">
         <v>800000</v>
@@ -8307,7 +8894,7 @@
     </row>
     <row r="55" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B55" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C55">
         <v>900000</v>
@@ -8318,7 +8905,7 @@
     </row>
     <row r="56" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B56" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C56">
         <v>1000000</v>
@@ -8329,7 +8916,7 @@
     </row>
     <row r="57" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B57" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C57">
         <v>1200000</v>
@@ -8340,7 +8927,7 @@
     </row>
     <row r="58" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B58" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C58">
         <v>1400000</v>
@@ -8351,7 +8938,7 @@
     </row>
     <row r="59" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B59" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C59">
         <v>1600000</v>
@@ -8362,7 +8949,7 @@
     </row>
     <row r="60" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B60" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C60">
         <v>1800000</v>
@@ -8373,7 +8960,7 @@
     </row>
     <row r="61" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B61" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C61">
         <v>2000000</v>
@@ -8384,7 +8971,7 @@
     </row>
     <row r="62" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B62" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C62">
         <v>200</v>
@@ -8395,7 +8982,7 @@
     </row>
     <row r="63" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B63" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C63">
         <v>400</v>
@@ -8406,7 +8993,7 @@
     </row>
     <row r="64" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B64" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C64">
         <v>1000</v>
@@ -8417,7 +9004,7 @@
     </row>
     <row r="65" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B65" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C65">
         <v>2000</v>
@@ -8428,7 +9015,7 @@
     </row>
     <row r="66" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B66" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C66">
         <v>4000</v>
@@ -8439,7 +9026,7 @@
     </row>
     <row r="67" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B67" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C67">
         <v>10000</v>
@@ -8450,7 +9037,7 @@
     </row>
     <row r="68" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B68" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C68">
         <v>20000</v>
@@ -8461,7 +9048,7 @@
     </row>
     <row r="69" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B69" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C69">
         <v>40000</v>
@@ -8472,7 +9059,7 @@
     </row>
     <row r="70" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B70" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C70">
         <v>80000</v>
@@ -8483,7 +9070,7 @@
     </row>
     <row r="71" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B71" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C71">
         <v>100000</v>
@@ -8494,7 +9081,7 @@
     </row>
     <row r="72" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B72" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C72">
         <v>150000</v>
@@ -8505,7 +9092,7 @@
     </row>
     <row r="73" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B73" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C73">
         <v>200000</v>
@@ -8516,7 +9103,7 @@
     </row>
     <row r="74" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B74" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C74">
         <v>250000</v>
@@ -8527,7 +9114,7 @@
     </row>
     <row r="75" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B75" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C75">
         <v>300000</v>
@@ -8538,7 +9125,7 @@
     </row>
     <row r="76" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B76" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C76">
         <v>350000</v>
@@ -8549,7 +9136,7 @@
     </row>
     <row r="77" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B77" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C77">
         <v>400000</v>
@@ -8560,7 +9147,7 @@
     </row>
     <row r="78" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B78" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C78">
         <v>500000</v>
@@ -8571,7 +9158,7 @@
     </row>
     <row r="79" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B79" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C79">
         <v>600000</v>
@@ -8582,7 +9169,7 @@
     </row>
     <row r="80" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B80" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C80">
         <v>700000</v>
@@ -8593,7 +9180,7 @@
     </row>
     <row r="81" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B81" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C81">
         <v>800000</v>
@@ -8604,7 +9191,7 @@
     </row>
     <row r="82" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B82" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C82">
         <v>900000</v>
@@ -8615,7 +9202,7 @@
     </row>
     <row r="83" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B83" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C83">
         <v>1000000</v>
@@ -8626,7 +9213,7 @@
     </row>
     <row r="84" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B84" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C84">
         <v>1200000</v>
@@ -8637,7 +9224,7 @@
     </row>
     <row r="85" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B85" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C85">
         <v>1400000</v>
@@ -8648,7 +9235,7 @@
     </row>
     <row r="86" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B86" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C86">
         <v>1600000</v>
@@ -8659,7 +9246,7 @@
     </row>
     <row r="87" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B87" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C87">
         <v>1800000</v>
@@ -8670,7 +9257,7 @@
     </row>
     <row r="88" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B88" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C88">
         <v>2000000</v>

</xml_diff>